<commit_message>
Cambiar Realizado en la fecha  2026-04-19 15:21:51
</commit_message>
<xml_diff>
--- a/Requisitos para aprobar el semillero/3 - Plan de Trabajo/Plan de trabajo FUAA.xlsx
+++ b/Requisitos para aprobar el semillero/3 - Plan de Trabajo/Plan de trabajo FUAA.xlsx
@@ -7,7 +7,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B57D8D79-EC94-475A-BBD7-D16BE7DAF5FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B8F1564-4FFB-4082-A4C7-876B12A487DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" activeTab="0"/>
   </bookViews>
@@ -126,8 +126,11 @@
         <color rgb="FFFFFFFF"/>
         <family val="2"/>
       </rPr>
-      <t>META
-NUMÉRICA</t>
+      <t xml:space="preserve">META
+</t>
+    </r>
+    <r>
+      <t>NUMÉRICA</t>
     </r>
   </si>
   <si>
@@ -154,8 +157,11 @@
         <color rgb="FFFFFFFF"/>
         <family val="2"/>
       </rPr>
-      <t>ENTREGABLE
-VERIF.</t>
+      <t xml:space="preserve">ENTREGABLE
+</t>
+    </r>
+    <r>
+      <t>VERIF.</t>
     </r>
   </si>
   <si>
@@ -173,8 +179,11 @@
         <color rgb="FFFFFFFF"/>
         <family val="2"/>
       </rPr>
-      <t>APROBADO
-POR</t>
+      <t xml:space="preserve">APROBADO
+</t>
+    </r>
+    <r>
+      <t>POR</t>
     </r>
   </si>
   <si>
@@ -384,7 +393,10 @@
         <family val="2"/>
       </rPr>
       <t>Escriba libremente los nombres de los integrantes a cargo.
-Para múltiples responsables sepárelos por coma.
+P</t>
+    </r>
+    <r>
+      <t>ara múltiples responsables sepárelos por coma.
 Ej: Juan Diego, David Ospina</t>
     </r>
   </si>
@@ -423,8 +435,11 @@
         <color rgb="FF1A1A1A"/>
         <family val="2"/>
       </rPr>
-      <t>Avance como decimal entre 0 y 1. La barra verde crece automáticamente.
-Ejemplo: escriba 0.75 para representar el 75%.</t>
+      <t xml:space="preserve">Avance como decimal entre 0 y 1. La barra verde crece automáticamente.
+</t>
+    </r>
+    <r>
+      <t>Ejemplo: escriba 0.75 para representar el 75%.</t>
     </r>
   </si>
   <si>
@@ -438,8 +453,11 @@
         <color rgb="FF1A1A1A"/>
         <family val="2"/>
       </rPr>
-      <t>Estado actual de la actividad. Menú desplegable.
-El color se asigna automáticamente.</t>
+      <t xml:space="preserve">Estado actual de la actividad. Menú desplegable.
+</t>
+    </r>
+    <r>
+      <t>El color se asigna automáticamente.</t>
     </r>
   </si>
   <si>
@@ -452,10 +470,10 @@
         <family val="2"/>
       </rPr>
       <t>✅ Completado · ⏳ En proceso
-📅 Pendiente · 🔴 Críti</t>
+📅</t>
     </r>
     <r>
-      <t>co</t>
+      <t xml:space="preserve"> Pendiente · 🔴 Crítico</t>
     </r>
   </si>
   <si>
@@ -512,6 +530,13 @@
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="14.00"/>
+      <b/>
+      <color rgb="FF1A1A1A"/>
+      <family val="2"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -536,7 +561,8 @@
     <font>
       <name val="Arial"/>
       <sz val="9.00"/>
-      <color rgb="FFEDF7D6"/>
+      <b/>
+      <color rgb="FF1A1A1A"/>
       <family val="2"/>
     </font>
     <font>
@@ -547,8 +573,22 @@
     </font>
     <font>
       <name val="Arial"/>
+      <sz val="22.00"/>
+      <b/>
+      <color rgb="FF1A1A1A"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="8.00"/>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="9.00"/>
-      <i/>
+      <b/>
       <color rgb="FF5A8500"/>
       <family val="2"/>
     </font>
@@ -567,28 +607,21 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="20.00"/>
+      <sz val="12.00"/>
       <b/>
       <color rgb="FFFFFFFF"/>
       <family val="2"/>
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="8.00"/>
+      <sz val="10.00"/>
       <b/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF5A8500"/>
       <family val="2"/>
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="14.00"/>
-      <b/>
-      <color rgb="FF1A1A1A"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10.00"/>
+      <sz val="22.00"/>
       <b/>
       <color rgb="FFFFFFFF"/>
       <family val="2"/>
@@ -602,30 +635,15 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="9.00"/>
+      <sz val="20.00"/>
       <b/>
-      <color rgb="FF1A1A1A"/>
+      <color rgb="FFFFFFFF"/>
       <family val="2"/>
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="22.00"/>
-      <b/>
-      <color rgb="FF1A1A1A"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10.00"/>
-      <b/>
-      <color rgb="FF5A8500"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="12.00"/>
-      <b/>
-      <color rgb="FFFFFFFF"/>
+      <sz val="9.00"/>
+      <color rgb="FFEDF7D6"/>
       <family val="2"/>
     </font>
     <font>
@@ -637,25 +655,31 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="22.00"/>
+      <sz val="9.00"/>
+      <i/>
+      <color rgb="FF5A8500"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10.00"/>
       <b/>
       <color rgb="FFFFFFFF"/>
       <family val="2"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="9.00"/>
-      <b/>
-      <color rgb="FF5A8500"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="36">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -671,7 +695,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF5A8500"/>
+        <fgColor rgb="FFEDF7D6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -683,7 +707,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF5A8500"/>
+        <fgColor rgb="FFFFFFFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -695,7 +719,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEDF7D6"/>
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF80BC00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -719,7 +749,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF5A8500"/>
+        <fgColor rgb="FFEDF7D6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -731,6 +761,36 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFEDF7D6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDF7D6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5A8500"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF80BC00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF80BC00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF5A8500"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -749,7 +809,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FF80BC00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5A8500"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5A8500"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -767,13 +839,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEDF7D6"/>
+        <fgColor rgb="FFFFFFFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF80BC00"/>
+        <fgColor rgb="FFB8DC6E"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -785,13 +857,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF80BC00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFB8DC6E"/>
+        <fgColor rgb="FFEDF7D6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -801,68 +867,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF80BC00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEDF7D6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEDF7D6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEDF7D6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF80BC00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF80BC00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="24">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -886,17 +892,62 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FF80BC00"/>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
       </left>
-      <right style="medium">
-        <color rgb="FF80BC00"/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
       </right>
-      <top style="medium">
-        <color rgb="FF80BC00"/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
       </top>
-      <bottom style="medium">
-        <color rgb="FF80BC00"/>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1002,21 +1053,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF80BC00"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF80BC00"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF80BC00"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF80BC00"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1111,62 +1147,17 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
+      <left style="medium">
+        <color rgb="FF80BC00"/>
       </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
+      <right style="medium">
+        <color rgb="FF80BC00"/>
       </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
+      <top style="medium">
+        <color rgb="FF80BC00"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
+      <bottom style="medium">
+        <color rgb="FF80BC00"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1200,216 +1191,192 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="36">
+  <cellStyleXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf fontId="1" applyFont="1" fillId="2" applyFill="1" borderId="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf fontId="2" applyFont="1" fillId="3" applyFill="1" borderId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center" wrapText="1"/>
+    </xf>
+    <xf fontId="3" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf fontId="4" applyFont="1" fillId="5" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left" wrapText="1"/>
     </xf>
-    <xf fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf fontId="5" applyFont="1" fillId="6" applyFill="1" borderId="3" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf fontId="2" applyFont="1" fillId="4" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" applyFont="1" fillId="7" applyFill="1" borderId="4" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="6" applyFont="1" fillId="8" applyFill="1" borderId="5" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf fontId="7" applyFont="1" fillId="9" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf fontId="8" applyFont="1" fillId="10" applyFill="1" borderId="6" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf fontId="9" applyFont="1" fillId="11" applyFill="1" borderId="7" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="6" applyFont="1" fillId="12" applyFill="1" borderId="8" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf fontId="10" applyFont="1" fillId="13" applyFill="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf fontId="3" applyFont="1" fillId="5" applyFill="1" borderId="3" applyBorder="1" applyAlignment="1">
+    <xf fontId="11" applyFont="1"/>
+    <xf fontId="2" applyFont="1" fillId="14" applyFill="1" borderId="9" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left" wrapText="1"/>
     </xf>
-    <xf fontId="4" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+    <xf fontId="12" applyFont="1" fillId="15" applyFill="1" borderId="10" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf fontId="1" applyFont="1" fillId="7" applyFill="1" borderId="4" applyBorder="1" applyAlignment="1">
+    <xf fontId="13" applyFont="1" fillId="16" applyFill="1" borderId="11" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf fontId="9" applyFont="1" fillId="17" applyFill="1" borderId="12" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf fontId="8" applyFont="1" fillId="18" applyFill="1" borderId="13" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf fontId="11" applyFont="1" fillId="19" applyFill="1"/>
+    <xf fontId="14" applyFont="1" fillId="20" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf fontId="11" applyFont="1" fillId="21" applyFill="1" borderId="14" applyBorder="1"/>
+    <xf fontId="15" applyFont="1" fillId="22" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf fontId="3" applyFont="1" fillId="23" applyFill="1" borderId="15" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf fontId="16" applyFont="1" fillId="24" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf fontId="17" applyFont="1" fillId="25" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf fontId="18" applyFont="1" fillId="26" applyFill="1" borderId="16" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center" wrapText="1"/>
     </xf>
-    <xf fontId="5" applyFont="1" fillId="8" applyFill="1" borderId="5" applyBorder="1" applyAlignment="1">
+    <xf fontId="9" applyFont="1" fillId="27" applyFill="1" borderId="17" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="19" applyFont="1" fillId="28" applyFill="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left"/>
     </xf>
-    <xf fontId="3" applyFont="1" fillId="9" applyFill="1" borderId="6" applyBorder="1" applyAlignment="1">
+    <xf fontId="4" applyFont="1" fillId="29" applyFill="1" borderId="18" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left" wrapText="1"/>
     </xf>
-    <xf fontId="6" applyFont="1" fillId="10" applyFill="1" borderId="7" applyBorder="1" applyAlignment="1">
+    <xf fontId="11" applyFont="1" fillId="30" applyFill="1"/>
+    <xf fontId="20" applyFont="1" fillId="31" applyFill="1" borderId="19" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf fontId="19" applyFont="1" fillId="32" applyFill="1" borderId="20" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left" wrapText="1"/>
     </xf>
-    <xf fontId="7" applyFont="1" fillId="11" applyFill="1" applyAlignment="1">
+    <xf fontId="2" applyFont="1" fillId="33" applyFill="1" borderId="21" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center" wrapText="1"/>
+    </xf>
+  </cellStyleXfs>
+  <cellXfs count="34">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf xfId="19" quotePrefix="0" pivotButton="0" fontId="11" applyFont="1" fillId="19" applyFill="1"/>
+    <xf xfId="20" quotePrefix="0" pivotButton="0" fontId="14" applyFont="1" fillId="20" applyFill="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf fontId="8" applyFont="1" fillId="12" applyFill="1" borderId="8" applyBorder="1"/>
-    <xf fontId="9" applyFont="1" fillId="13" applyFill="1" applyAlignment="1">
+    <xf xfId="8" quotePrefix="0" pivotButton="0" fontId="7" applyFont="1" fillId="9" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf xfId="3" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf fontId="10" applyFont="1" fillId="14" applyFill="1" borderId="9" applyBorder="1" applyAlignment="1">
+    <xf xfId="25" quotePrefix="0" pivotButton="0" fontId="17" applyFont="1" fillId="25" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf xfId="28" quotePrefix="0" pivotButton="0" fontId="19" applyFont="1" fillId="28" applyFill="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left"/>
     </xf>
-    <xf fontId="11" applyFont="1" fillId="15" applyFill="1" applyAlignment="1">
+    <xf xfId="12" quotePrefix="0" pivotButton="0" fontId="10" applyFont="1" fillId="13" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf xfId="18" quotePrefix="0" pivotButton="0" fontId="8" applyFont="1" fillId="18" applyFill="1" borderId="13" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left"/>
     </xf>
-    <xf fontId="12" applyFont="1" fillId="16" applyFill="1" borderId="10" applyBorder="1" applyAlignment="1">
+    <xf xfId="17" quotePrefix="0" pivotButton="0" fontId="9" applyFont="1" fillId="17" applyFill="1" borderId="12" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf xfId="9" quotePrefix="0" pivotButton="0" fontId="8" applyFont="1" fillId="10" applyFill="1" borderId="6" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf xfId="5" quotePrefix="0" pivotButton="0" fontId="5" applyFont="1" fillId="6" applyFill="1" borderId="3" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf fontId="13" applyFont="1" fillId="17" applyFill="1" applyAlignment="1">
+    <xf xfId="30" quotePrefix="0" pivotButton="0" fontId="11" applyFont="1" fillId="30" applyFill="1"/>
+    <xf xfId="26" quotePrefix="0" pivotButton="0" fontId="18" applyFont="1" fillId="26" applyFill="1" borderId="16" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="33" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" fillId="33" applyFill="1" borderId="21" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="6" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" fillId="7" applyFill="1" borderId="4" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="2" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" fillId="3" applyFill="1" borderId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="14" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" fillId="14" applyFill="1" borderId="9" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="31" quotePrefix="0" pivotButton="0" fontId="20" applyFont="1" fillId="31" applyFill="1" borderId="19" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf xfId="15" quotePrefix="0" pivotButton="0" fontId="12" applyFont="1" fillId="15" applyFill="1" borderId="10" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf xfId="21" quotePrefix="0" pivotButton="0" fontId="11" applyFont="1" fillId="21" applyFill="1" borderId="14" applyBorder="1"/>
+    <xf xfId="13" quotePrefix="0" pivotButton="0" fontId="11" applyFont="1"/>
+    <xf xfId="24" quotePrefix="0" pivotButton="0" fontId="16" applyFont="1" fillId="24" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf xfId="1" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left"/>
     </xf>
-    <xf fontId="14" applyFont="1" fillId="18" applyFill="1" borderId="11" applyBorder="1" applyAlignment="1">
+    <xf xfId="22" quotePrefix="0" pivotButton="0" fontId="15" applyFont="1" fillId="22" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf xfId="10" quotePrefix="0" pivotButton="0" fontId="9" applyFont="1" fillId="11" applyFill="1" borderId="7" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="4" quotePrefix="0" pivotButton="0" fontId="4" applyFont="1" fillId="5" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="27" quotePrefix="0" pivotButton="0" fontId="9" applyFont="1" fillId="27" applyFill="1" borderId="17" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="29" quotePrefix="0" pivotButton="0" fontId="4" applyFont="1" fillId="29" applyFill="1" borderId="18" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="32" quotePrefix="0" pivotButton="0" fontId="19" applyFont="1" fillId="32" applyFill="1" borderId="20" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="23" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1" fillId="23" applyFill="1" borderId="15" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf fontId="15" applyFont="1" fillId="19" applyFill="1" applyAlignment="1">
+    <xf xfId="11" quotePrefix="0" pivotButton="0" fontId="6" applyFont="1" fillId="12" applyFill="1" borderId="8" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left"/>
     </xf>
-    <xf fontId="16" applyFont="1" fillId="20" applyFill="1" borderId="12" applyBorder="1" applyAlignment="1">
+    <xf xfId="7" quotePrefix="0" pivotButton="0" fontId="6" applyFont="1" fillId="8" applyFill="1" borderId="5" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left"/>
     </xf>
-    <xf fontId="17" applyFont="1" fillId="21" applyFill="1" borderId="13" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf fontId="18" applyFont="1" fillId="22" applyFill="1" borderId="14" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf fontId="19" applyFont="1" fillId="23" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf fontId="8" applyFont="1" fillId="24" applyFill="1"/>
-    <xf fontId="20" applyFont="1" fillId="25" applyFill="1" borderId="15" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf fontId="10" applyFont="1" fillId="26" applyFill="1" borderId="16" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf fontId="1" applyFont="1" fillId="27" applyFill="1" borderId="17" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf fontId="20" applyFont="1" fillId="28" applyFill="1" borderId="18" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf fontId="20" applyFont="1" fillId="29" applyFill="1" borderId="19" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf fontId="1" applyFont="1" fillId="30" applyFill="1" borderId="20" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf fontId="17" applyFont="1" fillId="31" applyFill="1" borderId="21" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf fontId="6" applyFont="1" fillId="32" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf fontId="1" applyFont="1" fillId="33" applyFill="1" borderId="22" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf fontId="8" applyFont="1" fillId="34" applyFill="1"/>
-    <xf fontId="8" applyFont="1"/>
-    <xf fontId="5" applyFont="1" fillId="35" applyFill="1" borderId="23" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-  </cellStyleXfs>
-  <cellXfs count="35">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf xfId="33" quotePrefix="0" pivotButton="0" fontId="8" applyFont="1" fillId="34" applyFill="1"/>
-    <xf xfId="22" quotePrefix="0" pivotButton="0" fontId="19" applyFont="1" fillId="23" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf xfId="18" quotePrefix="0" pivotButton="0" fontId="15" applyFont="1" fillId="19" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf xfId="2" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf xfId="5" quotePrefix="0" pivotButton="0" fontId="4" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf xfId="31" quotePrefix="0" pivotButton="0" fontId="6" applyFont="1" fillId="32" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf xfId="10" quotePrefix="0" pivotButton="0" fontId="7" applyFont="1" fillId="11" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf xfId="13" quotePrefix="0" pivotButton="0" fontId="10" applyFont="1" fillId="14" applyFill="1" borderId="9" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf xfId="28" quotePrefix="0" pivotButton="0" fontId="20" applyFont="1" fillId="29" applyFill="1" borderId="19" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf xfId="25" quotePrefix="0" pivotButton="0" fontId="10" applyFont="1" fillId="26" applyFill="1" borderId="16" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf xfId="17" quotePrefix="0" pivotButton="0" fontId="14" applyFont="1" fillId="18" applyFill="1" borderId="11" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf xfId="23" quotePrefix="0" pivotButton="0" fontId="8" applyFont="1" fillId="24" applyFill="1"/>
-    <xf xfId="21" quotePrefix="0" pivotButton="0" fontId="18" applyFont="1" fillId="22" applyFill="1" borderId="14" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="6" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="7" applyFill="1" borderId="4" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="32" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="33" applyFill="1" borderId="22" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="29" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="30" applyFill="1" borderId="20" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="26" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="27" applyFill="1" borderId="17" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="1" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="2" applyFill="1" borderId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="15" quotePrefix="0" pivotButton="0" fontId="12" applyFont="1" fillId="16" applyFill="1" borderId="10" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf xfId="30" quotePrefix="0" pivotButton="0" fontId="17" applyFont="1" fillId="31" applyFill="1" borderId="21" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf xfId="11" quotePrefix="0" pivotButton="0" fontId="8" applyFont="1" fillId="12" applyFill="1" borderId="8" applyBorder="1"/>
-    <xf xfId="34" quotePrefix="0" pivotButton="0" fontId="8" applyFont="1"/>
-    <xf xfId="12" quotePrefix="0" pivotButton="0" fontId="9" applyFont="1" fillId="13" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf xfId="14" quotePrefix="0" pivotButton="0" fontId="11" applyFont="1" fillId="15" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf xfId="16" quotePrefix="0" pivotButton="0" fontId="13" applyFont="1" fillId="17" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf xfId="27" quotePrefix="0" pivotButton="0" fontId="20" applyFont="1" fillId="28" applyFill="1" borderId="18" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="8" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1" fillId="9" applyFill="1" borderId="6" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="24" quotePrefix="0" pivotButton="0" fontId="20" applyFont="1" fillId="25" applyFill="1" borderId="15" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="4" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1" fillId="5" applyFill="1" borderId="3" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="9" quotePrefix="0" pivotButton="0" fontId="6" applyFont="1" fillId="10" applyFill="1" borderId="7" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="3" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" fillId="4" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf xfId="7" quotePrefix="0" pivotButton="0" fontId="5" applyFont="1" fillId="8" applyFill="1" borderId="5" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf xfId="35" quotePrefix="0" pivotButton="0" fontId="5" applyFont="1" fillId="35" applyFill="1" borderId="23" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf xfId="19" quotePrefix="0" pivotButton="0" fontId="16" applyFont="1" fillId="20" applyFill="1" borderId="12" applyBorder="1" applyAlignment="1">
+    <xf xfId="16" quotePrefix="0" pivotButton="0" fontId="13" applyFont="1" fillId="16" applyFill="1" borderId="11" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1977,7 +1944,7 @@
       <c r="K10" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="L10" s="16">
+      <c r="L10" s="14">
         <v>1</v>
       </c>
       <c r="M10" s="14" t="s">
@@ -1991,13 +1958,13 @@
       </c>
     </row>
     <row r="11" ht="15.00" customHeight="true">
-      <c r="A11" s="17">
+      <c r="A11" s="16">
         <v>2</v>
       </c>
       <c r="B11" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="17" t="s">
         <v>47</v>
       </c>
       <c r="D11" s="15" t="s">
@@ -2006,7 +1973,7 @@
       <c r="E11" s="14">
         <v>3</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="17" t="s">
         <v>48</v>
       </c>
       <c r="G11" s="14">
@@ -2018,13 +1985,13 @@
       <c r="I11" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="J11" s="17" t="s">
+      <c r="J11" s="16" t="s">
         <v>42</v>
       </c>
       <c r="K11" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="L11" s="16">
+      <c r="L11" s="14">
         <v>1</v>
       </c>
       <c r="M11" s="14" t="s">
@@ -2071,7 +2038,7 @@
       <c r="K12" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="L12" s="16">
+      <c r="L12" s="14">
         <v>1</v>
       </c>
       <c r="M12" s="14" t="s">
@@ -2085,13 +2052,13 @@
       </c>
     </row>
     <row r="13" ht="15.00" customHeight="true">
-      <c r="A13" s="17">
+      <c r="A13" s="16">
         <v>4</v>
       </c>
       <c r="B13" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="17" t="s">
         <v>51</v>
       </c>
       <c r="D13" s="15" t="s">
@@ -2100,7 +2067,7 @@
       <c r="E13" s="14">
         <v>3</v>
       </c>
-      <c r="F13" s="18" t="s">
+      <c r="F13" s="17" t="s">
         <v>52</v>
       </c>
       <c r="G13" s="14">
@@ -2118,7 +2085,7 @@
       <c r="K13" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="L13" s="16">
+      <c r="L13" s="14">
         <v>1</v>
       </c>
       <c r="M13" s="14" t="s">
@@ -2159,13 +2126,13 @@
       <c r="I14" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="J14" s="17" t="s">
+      <c r="J14" s="16" t="s">
         <v>42</v>
       </c>
       <c r="K14" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="L14" s="16">
+      <c r="L14" s="14">
         <v>1</v>
       </c>
       <c r="M14" s="14" t="s">
@@ -2179,13 +2146,13 @@
       </c>
     </row>
     <row r="15" ht="15.00" customHeight="true">
-      <c r="A15" s="17">
+      <c r="A15" s="16">
         <v>6</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="17" t="s">
         <v>55</v>
       </c>
       <c r="D15" s="15" t="s">
@@ -2194,7 +2161,7 @@
       <c r="E15" s="14">
         <v>3</v>
       </c>
-      <c r="F15" s="18" t="s">
+      <c r="F15" s="17" t="s">
         <v>56</v>
       </c>
       <c r="G15" s="14">
@@ -2212,7 +2179,7 @@
       <c r="K15" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="L15" s="16">
+      <c r="L15" s="14">
         <v>1</v>
       </c>
       <c r="M15" s="14" t="s">
@@ -2259,7 +2226,7 @@
       <c r="K16" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="L16" s="16">
+      <c r="L16" s="14">
         <v>1</v>
       </c>
       <c r="M16" s="14" t="s">
@@ -2273,29 +2240,29 @@
       </c>
     </row>
     <row r="17" ht="21.75" customHeight="true">
-      <c r="A17" s="17">
+      <c r="A17" s="16">
         <v>10</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="17" t="s">
         <v>59</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="E17" s="17"/>
-      <c r="F17" s="18" t="s">
+      <c r="E17" s="16"/>
+      <c r="F17" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="G17" s="17" t="s">
+      <c r="G17" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="H17" s="17" t="s">
+      <c r="H17" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="I17" s="17" t="s">
+      <c r="I17" s="16" t="s">
         <v>63</v>
       </c>
       <c r="J17" s="14" t="s">
@@ -2304,10 +2271,10 @@
       <c r="K17" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="L17" s="17">
+      <c r="L17" s="16">
         <v>0.6</v>
       </c>
-      <c r="M17" s="17" t="s">
+      <c r="M17" s="16" t="s">
         <v>64</v>
       </c>
       <c r="N17" s="14"/>
@@ -2341,7 +2308,7 @@
       <c r="I18" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="J18" s="17" t="s">
+      <c r="J18" s="16" t="s">
         <v>42</v>
       </c>
       <c r="K18" s="14" t="s">
@@ -2359,29 +2326,29 @@
       </c>
     </row>
     <row r="19" ht="21.75" customHeight="true">
-      <c r="A19" s="17">
+      <c r="A19" s="16">
         <v>12</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="C19" s="18" t="s">
+      <c r="C19" s="17" t="s">
         <v>67</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="E19" s="17"/>
-      <c r="F19" s="18" t="s">
+      <c r="E19" s="16"/>
+      <c r="F19" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="G19" s="17" t="s">
+      <c r="G19" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="H19" s="17" t="s">
+      <c r="H19" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="I19" s="17" t="s">
+      <c r="I19" s="16" t="s">
         <v>63</v>
       </c>
       <c r="J19" s="14" t="s">
@@ -2390,10 +2357,10 @@
       <c r="K19" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="L19" s="17">
+      <c r="L19" s="16">
         <v>0.4</v>
       </c>
-      <c r="M19" s="17" t="s">
+      <c r="M19" s="16" t="s">
         <v>64</v>
       </c>
       <c r="N19" s="14"/>
@@ -2445,41 +2412,41 @@
       </c>
     </row>
     <row r="21" ht="21.75" customHeight="true">
-      <c r="A21" s="17">
+      <c r="A21" s="16">
         <v>14</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="C21" s="18" t="s">
+      <c r="C21" s="17" t="s">
         <v>73</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="E21" s="17"/>
-      <c r="F21" s="18" t="s">
+      <c r="E21" s="16"/>
+      <c r="F21" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="G21" s="17" t="s">
+      <c r="G21" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="H21" s="17" t="s">
+      <c r="H21" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="I21" s="17" t="s">
+      <c r="I21" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="J21" s="17" t="s">
+      <c r="J21" s="16" t="s">
         <v>42</v>
       </c>
       <c r="K21" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="L21" s="17">
+      <c r="L21" s="16">
         <v>1</v>
       </c>
-      <c r="M21" s="17" t="s">
+      <c r="M21" s="16" t="s">
         <v>44</v>
       </c>
       <c r="N21" s="14"/>
@@ -2531,29 +2498,29 @@
       </c>
     </row>
     <row r="23" ht="21.75" customHeight="true">
-      <c r="A23" s="17">
+      <c r="A23" s="16">
         <v>16</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="C23" s="18" t="s">
+      <c r="C23" s="17" t="s">
         <v>75</v>
       </c>
       <c r="D23" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="E23" s="17"/>
-      <c r="F23" s="18" t="s">
+      <c r="E23" s="16"/>
+      <c r="F23" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="G23" s="17" t="s">
+      <c r="G23" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="H23" s="17" t="s">
+      <c r="H23" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="I23" s="17" t="s">
+      <c r="I23" s="16" t="s">
         <v>63</v>
       </c>
       <c r="J23" s="14" t="s">
@@ -2562,10 +2529,10 @@
       <c r="K23" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="L23" s="17">
+      <c r="L23" s="16">
         <v>1</v>
       </c>
-      <c r="M23" s="17" t="s">
+      <c r="M23" s="16" t="s">
         <v>44</v>
       </c>
       <c r="N23" s="14"/>
@@ -2599,7 +2566,7 @@
       <c r="I24" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="J24" s="17" t="s">
+      <c r="J24" s="16" t="s">
         <v>42</v>
       </c>
       <c r="K24" s="14" t="s">
@@ -2617,29 +2584,29 @@
       </c>
     </row>
     <row r="25" ht="21.75" customHeight="true">
-      <c r="A25" s="17">
+      <c r="A25" s="16">
         <v>18</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="B25" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="C25" s="18" t="s">
+      <c r="C25" s="17" t="s">
         <v>77</v>
       </c>
       <c r="D25" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="E25" s="17"/>
-      <c r="F25" s="18" t="s">
+      <c r="E25" s="16"/>
+      <c r="F25" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="G25" s="17" t="s">
+      <c r="G25" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="H25" s="17" t="s">
+      <c r="H25" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="I25" s="17" t="s">
+      <c r="I25" s="16" t="s">
         <v>63</v>
       </c>
       <c r="J25" s="14" t="s">
@@ -2648,10 +2615,10 @@
       <c r="K25" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="L25" s="17">
+      <c r="L25" s="16">
         <v>1</v>
       </c>
-      <c r="M25" s="17" t="s">
+      <c r="M25" s="16" t="s">
         <v>44</v>
       </c>
       <c r="N25" s="14"/>
@@ -2703,41 +2670,41 @@
       </c>
     </row>
     <row r="27" ht="21.75" customHeight="true">
-      <c r="A27" s="17">
+      <c r="A27" s="16">
         <v>20</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="B27" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="C27" s="18" t="s">
+      <c r="C27" s="17" t="s">
         <v>81</v>
       </c>
       <c r="D27" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="E27" s="17"/>
-      <c r="F27" s="18" t="s">
+      <c r="E27" s="16"/>
+      <c r="F27" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="G27" s="17" t="s">
+      <c r="G27" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="H27" s="17" t="s">
+      <c r="H27" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="I27" s="17" t="s">
+      <c r="I27" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="J27" s="17" t="s">
+      <c r="J27" s="16" t="s">
         <v>42</v>
       </c>
       <c r="K27" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="L27" s="17">
+      <c r="L27" s="16">
         <v>1</v>
       </c>
-      <c r="M27" s="17" t="s">
+      <c r="M27" s="16" t="s">
         <v>44</v>
       </c>
       <c r="N27" s="14"/>
@@ -2763,21 +2730,21 @@
       <c r="O28" s="15"/>
     </row>
     <row r="29" ht="21.75" customHeight="true">
-      <c r="A29" s="17"/>
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="18"/>
-      <c r="G29" s="17"/>
-      <c r="H29" s="17"/>
-      <c r="I29" s="17"/>
-      <c r="J29" s="17"/>
-      <c r="K29" s="17"/>
-      <c r="L29" s="17"/>
-      <c r="M29" s="17"/>
-      <c r="N29" s="17"/>
-      <c r="O29" s="18"/>
+      <c r="A29" s="16"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="16"/>
+      <c r="I29" s="16"/>
+      <c r="J29" s="16"/>
+      <c r="K29" s="16"/>
+      <c r="L29" s="16"/>
+      <c r="M29" s="16"/>
+      <c r="N29" s="16"/>
+      <c r="O29" s="17"/>
     </row>
     <row r="30" ht="21.75" customHeight="true">
       <c r="A30" s="14"/>
@@ -2797,21 +2764,21 @@
       <c r="O30" s="15"/>
     </row>
     <row r="31" ht="21.75" customHeight="true">
-      <c r="A31" s="17"/>
-      <c r="B31" s="18"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="18"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="18"/>
-      <c r="G31" s="17"/>
-      <c r="H31" s="17"/>
-      <c r="I31" s="17"/>
-      <c r="J31" s="17"/>
-      <c r="K31" s="17"/>
-      <c r="L31" s="17"/>
-      <c r="M31" s="17"/>
-      <c r="N31" s="17"/>
-      <c r="O31" s="18"/>
+      <c r="A31" s="16"/>
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="16"/>
+      <c r="H31" s="16"/>
+      <c r="I31" s="16"/>
+      <c r="J31" s="16"/>
+      <c r="K31" s="16"/>
+      <c r="L31" s="16"/>
+      <c r="M31" s="16"/>
+      <c r="N31" s="16"/>
+      <c r="O31" s="17"/>
     </row>
     <row r="32" ht="21.75" customHeight="true">
       <c r="A32" s="14"/>
@@ -2831,25 +2798,25 @@
       <c r="O32" s="15"/>
     </row>
     <row r="33" ht="25.50" customHeight="true">
-      <c r="A33" s="19" t="s">
+      <c r="A33" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="B33" s="19"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
-      <c r="F33" s="19"/>
-      <c r="G33" s="19"/>
-      <c r="H33" s="19"/>
-      <c r="I33" s="19"/>
-      <c r="J33" s="19"/>
-      <c r="K33" s="19"/>
-      <c r="L33" s="20">
+      <c r="B33" s="18"/>
+      <c r="C33" s="18"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="18"/>
+      <c r="G33" s="18"/>
+      <c r="H33" s="18"/>
+      <c r="I33" s="18"/>
+      <c r="J33" s="18"/>
+      <c r="K33" s="18"/>
+      <c r="L33" s="19">
         <f>=IFERROR(AVERAGEIF(L10:L32,"&gt;0",L10:L32),0)</f>
       </c>
-      <c r="M33" s="21"/>
-      <c r="N33" s="21"/>
-      <c r="O33" s="21"/>
+      <c r="M33" s="20"/>
+      <c r="N33" s="20"/>
+      <c r="O33" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -2884,47 +2851,47 @@
   <sheetFormatPr defaultRowHeight="15.00" customHeight="1" defaultColWidth="8.71"/>
   <sheetData>
     <row r="1" ht="15.00" customHeight="true">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="21" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="2" ht="15.00" customHeight="true">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="3" ht="15.00" customHeight="true">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="4" ht="15.00" customHeight="true">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="21" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="5" ht="15.00" customHeight="true">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="6" ht="15.00" customHeight="true">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="21" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="7" ht="15.00" customHeight="true">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="21" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="8" ht="15.00" customHeight="true">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="21" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="9" ht="15.00" customHeight="true">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="21" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2955,17 +2922,17 @@
       <c r="D1" s="1"/>
     </row>
     <row r="2" ht="49.50" customHeight="true">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
     </row>
     <row r="3" ht="19.50" customHeight="true">
-      <c r="A3" s="23"/>
+      <c r="A3" s="22"/>
       <c r="B3" s="6" t="s">
         <v>86</v>
       </c>
@@ -2973,12 +2940,12 @@
       <c r="D3" s="6"/>
     </row>
     <row r="4" ht="18.00" customHeight="true">
-      <c r="A4" s="23"/>
-      <c r="B4" s="25" t="s">
+      <c r="A4" s="22"/>
+      <c r="B4" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
     </row>
     <row r="5" ht="4.50" customHeight="true">
       <c r="A5" s="1"/>
@@ -2987,228 +2954,228 @@
       <c r="D5" s="1"/>
     </row>
     <row r="7" ht="27.75" customHeight="true">
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="18" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="8" ht="42.00" customHeight="true">
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="D8" s="27" t="s">
+      <c r="D8" s="26" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="9" ht="42.00" customHeight="true">
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="27" t="s">
         <v>23</v>
       </c>
       <c r="C9" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="D9" s="29" t="s">
+      <c r="D9" s="28" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="10" ht="42.00" customHeight="true">
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="D10" s="26" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="11" ht="42.00" customHeight="true">
-      <c r="B11" s="28" t="s">
+      <c r="B11" s="27" t="s">
         <v>25</v>
       </c>
       <c r="C11" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="D11" s="29" t="s">
+      <c r="D11" s="28" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="12" ht="42.00" customHeight="true">
-      <c r="B12" s="26" t="s">
+      <c r="B12" s="25" t="s">
         <v>99</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="D12" s="27" t="s">
+      <c r="D12" s="26" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="13" ht="42.00" customHeight="true">
-      <c r="B13" s="28" t="s">
+      <c r="B13" s="27" t="s">
         <v>27</v>
       </c>
       <c r="C13" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="D13" s="29" t="s">
+      <c r="D13" s="28" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="14" ht="42.00" customHeight="true">
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="25" t="s">
         <v>104</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="D14" s="27" t="s">
+      <c r="D14" s="26" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="15" ht="42.00" customHeight="true">
-      <c r="B15" s="28" t="s">
+      <c r="B15" s="27" t="s">
         <v>31</v>
       </c>
       <c r="C15" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="D15" s="29" t="s">
+      <c r="D15" s="28" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="16" ht="42.00" customHeight="true">
-      <c r="B16" s="26" t="s">
+      <c r="B16" s="25" t="s">
         <v>109</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="D16" s="27" t="s">
+      <c r="D16" s="26" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="17" ht="42.00" customHeight="true">
-      <c r="B17" s="28" t="s">
+      <c r="B17" s="27" t="s">
         <v>33</v>
       </c>
       <c r="C17" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="D17" s="29" t="s">
+      <c r="D17" s="28" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="18" ht="42.00" customHeight="true">
-      <c r="B18" s="26" t="s">
+      <c r="B18" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="C18" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="D18" s="27" t="s">
+      <c r="D18" s="26" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="19" ht="42.00" customHeight="true">
-      <c r="B19" s="28" t="s">
+      <c r="B19" s="27" t="s">
         <v>116</v>
       </c>
       <c r="C19" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="D19" s="29" t="s">
+      <c r="D19" s="28" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="20" ht="42.00" customHeight="true">
-      <c r="B20" s="26" t="s">
+      <c r="B20" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="C20" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="D20" s="27" t="s">
+      <c r="D20" s="26" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="22" ht="45.75" customHeight="true">
-      <c r="B22" s="30" t="s">
+      <c r="B22" s="29" t="s">
         <v>120</v>
       </c>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
     </row>
     <row r="24" ht="27.75" customHeight="true">
-      <c r="B24" s="31" t="s">
+      <c r="B24" s="30" t="s">
         <v>121</v>
       </c>
-      <c r="C24" s="31"/>
-      <c r="D24" s="31"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
     </row>
     <row r="25" ht="21.75" customHeight="true">
-      <c r="B25" s="32" t="s">
+      <c r="B25" s="31" t="s">
         <v>122</v>
       </c>
-      <c r="C25" s="32"/>
-      <c r="D25" s="32"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
     </row>
     <row r="26" ht="21.75" customHeight="true">
-      <c r="B26" s="33" t="s">
+      <c r="B26" s="32" t="s">
         <v>123</v>
       </c>
-      <c r="C26" s="33"/>
-      <c r="D26" s="33"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
     </row>
     <row r="27" ht="21.75" customHeight="true">
-      <c r="B27" s="32" t="s">
+      <c r="B27" s="31" t="s">
         <v>124</v>
       </c>
-      <c r="C27" s="32"/>
-      <c r="D27" s="32"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
     </row>
     <row r="28" ht="21.75" customHeight="true">
-      <c r="B28" s="33" t="s">
+      <c r="B28" s="32" t="s">
         <v>125</v>
       </c>
-      <c r="C28" s="33"/>
-      <c r="D28" s="33"/>
+      <c r="C28" s="32"/>
+      <c r="D28" s="32"/>
     </row>
     <row r="29" ht="21.75" customHeight="true">
-      <c r="B29" s="32" t="s">
+      <c r="B29" s="31" t="s">
         <v>126</v>
       </c>
-      <c r="C29" s="32"/>
-      <c r="D29" s="32"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="31"/>
     </row>
     <row r="30" ht="21.75" customHeight="true">
-      <c r="B30" s="33" t="s">
+      <c r="B30" s="32" t="s">
         <v>127</v>
       </c>
-      <c r="C30" s="33"/>
-      <c r="D30" s="33"/>
+      <c r="C30" s="32"/>
+      <c r="D30" s="32"/>
     </row>
     <row r="31" ht="21.75" customHeight="true">
-      <c r="B31" s="32" t="s">
+      <c r="B31" s="31" t="s">
         <v>128</v>
       </c>
-      <c r="C31" s="32"/>
-      <c r="D31" s="32"/>
+      <c r="C31" s="31"/>
+      <c r="D31" s="31"/>
     </row>
     <row r="32" ht="21.75" customHeight="true">
-      <c r="B32" s="34" t="s">
+      <c r="B32" s="33" t="s">
         <v>129</v>
       </c>
-      <c r="C32" s="34"/>
-      <c r="D32" s="34"/>
+      <c r="C32" s="33"/>
+      <c r="D32" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="14">

</xml_diff>

<commit_message>
Cambiar Realizado en la fecha  2026-04-19 16:10:28
</commit_message>
<xml_diff>
--- a/Requisitos para aprobar el semillero/3 - Plan de Trabajo/Plan de trabajo FUAA.xlsx
+++ b/Requisitos para aprobar el semillero/3 - Plan de Trabajo/Plan de trabajo FUAA.xlsx
@@ -7,7 +7,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B8F1564-4FFB-4082-A4C7-876B12A487DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41CEF1CC-C2BA-4836-9ED9-6EDB58B530CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" activeTab="0"/>
   </bookViews>
@@ -126,11 +126,8 @@
         <color rgb="FFFFFFFF"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">META
-</t>
-    </r>
-    <r>
-      <t>NUMÉRICA</t>
+      <t>META
+NUMÉRICA</t>
     </r>
   </si>
   <si>
@@ -157,11 +154,8 @@
         <color rgb="FFFFFFFF"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">ENTREGABLE
-</t>
-    </r>
-    <r>
-      <t>VERIF.</t>
+      <t>ENTREGABLE
+VERIF.</t>
     </r>
   </si>
   <si>
@@ -179,11 +173,8 @@
         <color rgb="FFFFFFFF"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">APROBADO
-</t>
-    </r>
-    <r>
-      <t>POR</t>
+      <t>APROBADO
+POR</t>
     </r>
   </si>
   <si>
@@ -393,10 +384,10 @@
         <family val="2"/>
       </rPr>
       <t>Escriba libremente los nombres de los integrantes a cargo.
-P</t>
+Pa</t>
     </r>
     <r>
-      <t>ara múltiples responsables sepárelos por coma.
+      <t>ra múltiples responsables sepárelos por coma.
 Ej: Juan Diego, David Ospina</t>
     </r>
   </si>
@@ -435,11 +426,8 @@
         <color rgb="FF1A1A1A"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">Avance como decimal entre 0 y 1. La barra verde crece automáticamente.
-</t>
-    </r>
-    <r>
-      <t>Ejemplo: escriba 0.75 para representar el 75%.</t>
+      <t>Avance como decimal entre 0 y 1. La barra verde crece automáticamente.
+Ejemplo: escriba 0.75 para representar el 75%.</t>
     </r>
   </si>
   <si>
@@ -453,11 +441,8 @@
         <color rgb="FF1A1A1A"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">Estado actual de la actividad. Menú desplegable.
-</t>
-    </r>
-    <r>
-      <t>El color se asigna automáticamente.</t>
+      <t>Estado actual de la actividad. Menú desplegable.
+El color se asigna automáticamente.</t>
     </r>
   </si>
   <si>
@@ -470,10 +455,10 @@
         <family val="2"/>
       </rPr>
       <t>✅ Completado · ⏳ En proceso
-📅</t>
+📅 Pendiente · 🔴 Crític</t>
     </r>
     <r>
-      <t xml:space="preserve"> Pendiente · 🔴 Crítico</t>
+      <t>o</t>
     </r>
   </si>
   <si>
@@ -533,15 +518,41 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="14.00"/>
-      <b/>
+      <sz val="8.00"/>
+      <i/>
+      <color rgb="FFB8DC6E"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10.00"/>
       <color rgb="FF1A1A1A"/>
       <family val="2"/>
     </font>
     <font>
       <name val="Arial"/>
       <sz val="9.00"/>
+      <b/>
+      <color rgb="FF5A8500"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.00"/>
+      <color rgb="FF000000"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9.00"/>
       <color rgb="FF1A1A1A"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9.00"/>
+      <b/>
+      <color rgb="FFFFFFFF"/>
       <family val="2"/>
     </font>
     <font>
@@ -553,9 +564,71 @@
     </font>
     <font>
       <name val="Arial"/>
+      <sz val="14.00"/>
+      <b/>
+      <color rgb="FF1A1A1A"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10.00"/>
+      <b/>
+      <color rgb="FF5A8500"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="8.00"/>
+      <i/>
+      <color rgb="FF666666"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="9.00"/>
       <i/>
       <color rgb="FF666666"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="8.00"/>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="20.00"/>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10.00"/>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="22.00"/>
+      <b/>
+      <color rgb="FF1A1A1A"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9.00"/>
+      <color rgb="FFEDF7D6"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9.00"/>
+      <i/>
+      <color rgb="FF5A8500"/>
       <family val="2"/>
     </font>
     <font>
@@ -567,42 +640,9 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="10.00"/>
-      <color rgb="FF1A1A1A"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <sz val="22.00"/>
       <b/>
-      <color rgb="FF1A1A1A"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="8.00"/>
-      <b/>
       <color rgb="FFFFFFFF"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="9.00"/>
-      <b/>
-      <color rgb="FF5A8500"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="8.00"/>
-      <i/>
-      <color rgb="FFB8DC6E"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.00"/>
-      <color rgb="FF000000"/>
       <family val="2"/>
     </font>
     <font>
@@ -612,61 +652,6 @@
       <color rgb="FFFFFFFF"/>
       <family val="2"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10.00"/>
-      <b/>
-      <color rgb="FF5A8500"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="22.00"/>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="8.00"/>
-      <i/>
-      <color rgb="FF666666"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="20.00"/>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="9.00"/>
-      <color rgb="FFEDF7D6"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="9.00"/>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="9.00"/>
-      <i/>
-      <color rgb="FF5A8500"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10.00"/>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="34">
     <fill>
@@ -674,6 +659,12 @@
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5A8500"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -683,7 +674,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEDF7D6"/>
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF80BC00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -695,7 +698,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEDF7D6"/>
+        <fgColor rgb="FF5A8500"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -707,7 +710,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FFEDF7D6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -725,7 +728,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF80BC00"/>
+        <fgColor rgb="FFEDF7D6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB8DC6E"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -737,7 +746,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEDF7D6"/>
+        <fgColor rgb="FF5A8500"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF80BC00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -755,7 +770,49 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFEDF7D6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5A8500"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF80BC00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5A8500"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5A8500"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -773,7 +830,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF5A8500"/>
+        <fgColor rgb="FFEDF7D6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -786,84 +849,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF80BC00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF5A8500"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF5A8500"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF80BC00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF5A8500"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF5A8500"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFB8DC6E"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF5A8500"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEDF7D6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -923,91 +908,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFCCCCCC"/>
+        <color rgb="FFB8DC6E"/>
       </left>
       <right style="thin">
-        <color rgb="FFCCCCCC"/>
+        <color rgb="FFB8DC6E"/>
       </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
+      <top style="medium">
+        <color rgb="FF80BC00"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
+      <bottom style="medium">
+        <color rgb="FF80BC00"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1072,17 +982,47 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FF80BC00"/>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
       </left>
-      <right style="medium">
-        <color rgb="FF80BC00"/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
       </right>
-      <top style="medium">
-        <color rgb="FF80BC00"/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
       </top>
-      <bottom style="medium">
-        <color rgb="FF80BC00"/>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1103,16 +1043,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFB8DC6E"/>
+        <color rgb="FFCCCCCC"/>
       </left>
       <right style="thin">
-        <color rgb="FFB8DC6E"/>
+        <color rgb="FFCCCCCC"/>
       </right>
-      <top style="medium">
-        <color rgb="FF80BC00"/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
       </top>
-      <bottom style="medium">
-        <color rgb="FF80BC00"/>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1128,36 +1068,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF80BC00"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF80BC00"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF80BC00"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF80BC00"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1191,192 +1101,267 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF80BC00"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF80BC00"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF80BC00"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF80BC00"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF80BC00"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF80BC00"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF80BC00"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF80BC00"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf fontId="2" applyFont="1" fillId="3" applyFill="1" borderId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left"/>
     </xf>
-    <xf fontId="2" applyFont="1" fillId="3" applyFill="1" borderId="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" applyFont="1" fillId="4" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="4" applyFont="1" fillId="5" applyFill="1"/>
+    <xf fontId="5" applyFont="1" fillId="6" applyFill="1" borderId="3" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="6" applyFont="1" fillId="7" applyFill="1" borderId="4" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center" wrapText="1"/>
     </xf>
-    <xf fontId="3" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf fontId="7" applyFont="1" fillId="8" applyFill="1" borderId="5" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf fontId="4" applyFont="1" fillId="5" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
+    <xf fontId="8" applyFont="1" fillId="9" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf fontId="9" applyFont="1" fillId="10" applyFill="1" borderId="6" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf fontId="10" applyFont="1" fillId="11" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf fontId="11" applyFont="1" fillId="12" applyFill="1" borderId="7" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left" wrapText="1"/>
     </xf>
-    <xf fontId="5" applyFont="1" fillId="6" applyFill="1" borderId="3" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" applyFont="1" fillId="13" applyFill="1" borderId="8" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="4" applyFont="1" fillId="14" applyFill="1"/>
+    <xf fontId="5" applyFont="1" fillId="15" applyFill="1" borderId="9" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center" wrapText="1"/>
+    </xf>
+    <xf fontId="12" applyFont="1" fillId="16" applyFill="1" borderId="10" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf fontId="12" applyFont="1" fillId="17" applyFill="1" borderId="11" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf fontId="4" applyFont="1" fillId="18" applyFill="1" borderId="12" applyBorder="1"/>
+    <xf fontId="3" applyFont="1" fillId="19" applyFill="1" borderId="13" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf fontId="3" applyFont="1" fillId="20" applyFill="1" borderId="14" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="7" applyFont="1" fillId="21" applyFill="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf fontId="2" applyFont="1" fillId="7" applyFill="1" borderId="4" applyBorder="1" applyAlignment="1">
+    <xf fontId="13" applyFont="1" fillId="22" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf fontId="14" applyFont="1" fillId="23" applyFill="1" borderId="15" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf fontId="4" applyFont="1"/>
+    <xf fontId="15" applyFont="1" fillId="24" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf fontId="16" applyFont="1" fillId="25" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf fontId="17" applyFont="1" fillId="26" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf fontId="5" applyFont="1" fillId="27" applyFill="1" borderId="16" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center" wrapText="1"/>
+    </xf>
+    <xf fontId="11" applyFont="1" fillId="28" applyFill="1" borderId="17" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left" wrapText="1"/>
     </xf>
-    <xf fontId="6" applyFont="1" fillId="8" applyFill="1" borderId="5" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" applyFont="1" fillId="29" applyFill="1" borderId="18" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left"/>
     </xf>
-    <xf fontId="7" applyFont="1" fillId="9" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf fontId="8" applyFont="1" fillId="10" applyFill="1" borderId="6" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf fontId="9" applyFont="1" fillId="11" applyFill="1" borderId="7" applyBorder="1" applyAlignment="1">
+    <xf fontId="17" applyFont="1" fillId="30" applyFill="1" borderId="19" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left" wrapText="1"/>
     </xf>
-    <xf fontId="6" applyFont="1" fillId="12" applyFill="1" borderId="8" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf fontId="10" applyFont="1" fillId="13" applyFill="1" applyAlignment="1">
+    <xf fontId="18" applyFont="1" fillId="31" applyFill="1" borderId="20" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf fontId="11" applyFont="1"/>
-    <xf fontId="2" applyFont="1" fillId="14" applyFill="1" borderId="9" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf fontId="12" applyFont="1" fillId="15" applyFill="1" borderId="10" applyBorder="1" applyAlignment="1">
+    <xf fontId="19" applyFont="1" fillId="32" applyFill="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf fontId="13" applyFont="1" fillId="16" applyFill="1" borderId="11" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf fontId="9" applyFont="1" fillId="17" applyFill="1" borderId="12" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf fontId="8" applyFont="1" fillId="18" applyFill="1" borderId="13" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf fontId="11" applyFont="1" fillId="19" applyFill="1"/>
-    <xf fontId="14" applyFont="1" fillId="20" applyFill="1" applyAlignment="1">
+    <xf fontId="20" applyFont="1" fillId="33" applyFill="1" borderId="21" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf fontId="11" applyFont="1" fillId="21" applyFill="1" borderId="14" applyBorder="1"/>
-    <xf fontId="15" applyFont="1" fillId="22" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf fontId="3" applyFont="1" fillId="23" applyFill="1" borderId="15" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf fontId="16" applyFont="1" fillId="24" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf fontId="17" applyFont="1" fillId="25" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf fontId="18" applyFont="1" fillId="26" applyFill="1" borderId="16" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf fontId="9" applyFont="1" fillId="27" applyFill="1" borderId="17" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf fontId="19" applyFont="1" fillId="28" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf fontId="4" applyFont="1" fillId="29" applyFill="1" borderId="18" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf fontId="11" applyFont="1" fillId="30" applyFill="1"/>
-    <xf fontId="20" applyFont="1" fillId="31" applyFill="1" borderId="19" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf fontId="19" applyFont="1" fillId="32" applyFill="1" borderId="20" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf fontId="2" applyFont="1" fillId="33" applyFill="1" borderId="21" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf xfId="19" quotePrefix="0" pivotButton="0" fontId="11" applyFont="1" fillId="19" applyFill="1"/>
-    <xf xfId="20" quotePrefix="0" pivotButton="0" fontId="14" applyFont="1" fillId="20" applyFill="1" applyAlignment="1">
+    <xf xfId="4" quotePrefix="0" pivotButton="0" fontId="4" applyFont="1" fillId="5" applyFill="1"/>
+    <xf xfId="32" quotePrefix="0" pivotButton="0" fontId="19" applyFont="1" fillId="32" applyFill="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf xfId="8" quotePrefix="0" pivotButton="0" fontId="7" applyFont="1" fillId="9" applyFill="1" applyAlignment="1">
+    <xf xfId="24" quotePrefix="0" pivotButton="0" fontId="15" applyFont="1" fillId="24" applyFill="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left"/>
     </xf>
-    <xf xfId="3" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf xfId="20" quotePrefix="0" pivotButton="0" fontId="7" applyFont="1" fillId="21" applyFill="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf xfId="25" quotePrefix="0" pivotButton="0" fontId="17" applyFont="1" fillId="25" applyFill="1" applyAlignment="1">
+    <xf xfId="25" quotePrefix="0" pivotButton="0" fontId="16" applyFont="1" fillId="25" applyFill="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf xfId="28" quotePrefix="0" pivotButton="0" fontId="19" applyFont="1" fillId="28" applyFill="1" applyAlignment="1">
+    <xf xfId="26" quotePrefix="0" pivotButton="0" fontId="17" applyFont="1" fillId="26" applyFill="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left"/>
     </xf>
-    <xf xfId="12" quotePrefix="0" pivotButton="0" fontId="10" applyFont="1" fillId="13" applyFill="1" applyAlignment="1">
+    <xf xfId="1" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf xfId="18" quotePrefix="0" pivotButton="0" fontId="8" applyFont="1" fillId="18" applyFill="1" borderId="13" applyBorder="1" applyAlignment="1">
+    <xf xfId="15" quotePrefix="0" pivotButton="0" fontId="12" applyFont="1" fillId="16" applyFill="1" borderId="10" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left"/>
     </xf>
-    <xf xfId="17" quotePrefix="0" pivotButton="0" fontId="9" applyFont="1" fillId="17" applyFill="1" borderId="12" applyBorder="1" applyAlignment="1">
+    <xf xfId="18" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1" fillId="19" applyFill="1" borderId="13" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left"/>
     </xf>
-    <xf xfId="9" quotePrefix="0" pivotButton="0" fontId="8" applyFont="1" fillId="10" applyFill="1" borderId="6" applyBorder="1" applyAlignment="1">
+    <xf xfId="16" quotePrefix="0" pivotButton="0" fontId="12" applyFont="1" fillId="17" applyFill="1" borderId="11" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left"/>
     </xf>
+    <xf xfId="31" quotePrefix="0" pivotButton="0" fontId="18" applyFont="1" fillId="31" applyFill="1" borderId="20" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf xfId="13" quotePrefix="0" pivotButton="0" fontId="4" applyFont="1" fillId="14" applyFill="1"/>
+    <xf xfId="6" quotePrefix="0" pivotButton="0" fontId="6" applyFont="1" fillId="7" applyFill="1" borderId="4" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="27" quotePrefix="0" pivotButton="0" fontId="5" applyFont="1" fillId="27" applyFill="1" borderId="16" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center" wrapText="1"/>
+    </xf>
     <xf xfId="5" quotePrefix="0" pivotButton="0" fontId="5" applyFont="1" fillId="6" applyFill="1" borderId="3" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="14" quotePrefix="0" pivotButton="0" fontId="5" applyFont="1" fillId="15" applyFill="1" borderId="9" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="12" quotePrefix="0" pivotButton="0" fontId="5" applyFont="1" fillId="13" applyFill="1" borderId="8" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="22" quotePrefix="0" pivotButton="0" fontId="14" applyFont="1" fillId="23" applyFill="1" borderId="15" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf xfId="30" quotePrefix="0" pivotButton="0" fontId="11" applyFont="1" fillId="30" applyFill="1"/>
-    <xf xfId="26" quotePrefix="0" pivotButton="0" fontId="18" applyFont="1" fillId="26" applyFill="1" borderId="16" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="33" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" fillId="33" applyFill="1" borderId="21" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="6" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" fillId="7" applyFill="1" borderId="4" applyBorder="1" applyAlignment="1">
+    <xf xfId="33" quotePrefix="0" pivotButton="0" fontId="20" applyFont="1" fillId="33" applyFill="1" borderId="21" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf xfId="17" quotePrefix="0" pivotButton="0" fontId="4" applyFont="1" fillId="18" applyFill="1" borderId="12" applyBorder="1"/>
+    <xf xfId="23" quotePrefix="0" pivotButton="0" fontId="4" applyFont="1"/>
+    <xf xfId="21" quotePrefix="0" pivotButton="0" fontId="13" applyFont="1" fillId="22" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf xfId="8" quotePrefix="0" pivotButton="0" fontId="8" applyFont="1" fillId="9" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf xfId="10" quotePrefix="0" pivotButton="0" fontId="10" applyFont="1" fillId="11" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
+    <xf xfId="19" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1" fillId="20" applyFill="1" borderId="14" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left" wrapText="1"/>
     </xf>
+    <xf xfId="28" quotePrefix="0" pivotButton="0" fontId="11" applyFont="1" fillId="28" applyFill="1" borderId="17" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="3" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1" fillId="4" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="11" quotePrefix="0" pivotButton="0" fontId="11" applyFont="1" fillId="12" applyFill="1" borderId="7" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="30" quotePrefix="0" pivotButton="0" fontId="17" applyFont="1" fillId="30" applyFill="1" borderId="19" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="7" quotePrefix="0" pivotButton="0" fontId="7" applyFont="1" fillId="8" applyFill="1" borderId="5" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf xfId="29" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" fillId="29" applyFill="1" borderId="18" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="left"/>
+    </xf>
     <xf xfId="2" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" fillId="3" applyFill="1" borderId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="14" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" fillId="14" applyFill="1" borderId="9" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="31" quotePrefix="0" pivotButton="0" fontId="20" applyFont="1" fillId="31" applyFill="1" borderId="19" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf xfId="15" quotePrefix="0" pivotButton="0" fontId="12" applyFont="1" fillId="15" applyFill="1" borderId="10" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf xfId="21" quotePrefix="0" pivotButton="0" fontId="11" applyFont="1" fillId="21" applyFill="1" borderId="14" applyBorder="1"/>
-    <xf xfId="13" quotePrefix="0" pivotButton="0" fontId="11" applyFont="1"/>
-    <xf xfId="24" quotePrefix="0" pivotButton="0" fontId="16" applyFont="1" fillId="24" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf xfId="1" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left"/>
     </xf>
-    <xf xfId="22" quotePrefix="0" pivotButton="0" fontId="15" applyFont="1" fillId="22" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf xfId="10" quotePrefix="0" pivotButton="0" fontId="9" applyFont="1" fillId="11" applyFill="1" borderId="7" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="4" quotePrefix="0" pivotButton="0" fontId="4" applyFont="1" fillId="5" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="27" quotePrefix="0" pivotButton="0" fontId="9" applyFont="1" fillId="27" applyFill="1" borderId="17" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="29" quotePrefix="0" pivotButton="0" fontId="4" applyFont="1" fillId="29" applyFill="1" borderId="18" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="32" quotePrefix="0" pivotButton="0" fontId="19" applyFont="1" fillId="32" applyFill="1" borderId="20" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="23" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1" fillId="23" applyFill="1" borderId="15" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf xfId="11" quotePrefix="0" pivotButton="0" fontId="6" applyFont="1" fillId="12" applyFill="1" borderId="8" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf xfId="7" quotePrefix="0" pivotButton="0" fontId="6" applyFont="1" fillId="8" applyFill="1" borderId="5" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf xfId="16" quotePrefix="0" pivotButton="0" fontId="13" applyFont="1" fillId="16" applyFill="1" borderId="11" applyBorder="1" applyAlignment="1">
+    <xf xfId="9" quotePrefix="0" pivotButton="0" fontId="9" applyFont="1" fillId="10" applyFill="1" borderId="6" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="left"/>
     </xf>
   </cellXfs>

</xml_diff>

<commit_message>
vault backup: 2026-05-09 12:06:57
</commit_message>
<xml_diff>
--- a/Requisitos para aprobar el semillero/3 - Plan de Trabajo/Plan de trabajo FUAA.xlsx
+++ b/Requisitos para aprobar el semillero/3 - Plan de Trabajo/Plan de trabajo FUAA.xlsx
@@ -1,44 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Areandina\Semillero\Docs\IA-DataFlow Hub - Semillero\Requisitos para aprobar el semillero\3 - Plan de Trabajo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A362F701-342B-44BA-9376-DDFA8980CCAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4BFDF2BC-2EF9-416D-894F-B055ED89C860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLAN DE TRABAJO" sheetId="1" r:id="rId1"/>
-    <sheet name="EQUIPO" sheetId="2" r:id="rId2" state="hidden"/>
+    <sheet name="EQUIPO" sheetId="2" state="hidden" r:id="rId2"/>
     <sheet name="INSTRUCTIVO" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="155">
   <si>
     <t>A</t>
   </si>
@@ -120,10 +109,10 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Arial"/>
-        <sz val="9.00"/>
-        <b/>
-        <color rgb="FFFFFFFF"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">META
@@ -131,9 +120,9 @@
     </r>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
-        <sz val="11.00"/>
-        <color rgb="FF000000"/>
         <family val="2"/>
       </rPr>
       <t>NUMÉRICA</t>
@@ -157,10 +146,10 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Arial"/>
-        <sz val="9.00"/>
-        <b/>
-        <color rgb="FFFFFFFF"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">ENTREGABLE
@@ -168,9 +157,9 @@
     </r>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
-        <sz val="11.00"/>
-        <color rgb="FF000000"/>
         <family val="2"/>
       </rPr>
       <t>VERIF.</t>
@@ -185,10 +174,10 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Arial"/>
-        <sz val="9.00"/>
-        <b/>
-        <color rgb="FFFFFFFF"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">APROBADO
@@ -196,9 +185,9 @@
     </r>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
-        <sz val="11.00"/>
-        <color rgb="FF000000"/>
         <family val="2"/>
       </rPr>
       <t>POR</t>
@@ -441,18 +430,32 @@
   <si>
     <r>
       <rPr>
+        <sz val="9"/>
+        <color rgb="FF1A1A1A"/>
         <rFont val="Arial"/>
-        <sz val="9.00"/>
-        <color rgb="FF1A1A1A"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">Escriba libremente los nombres de los integrantes a cargo.
 </t>
     </r>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>Pa</t>
     </r>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>ra múltiples responsables sepárelos por coma.
 Ej: Juan Diego, David Ospina</t>
     </r>
@@ -487,9 +490,9 @@
   <si>
     <r>
       <rPr>
+        <sz val="9"/>
+        <color rgb="FF1A1A1A"/>
         <rFont val="Arial"/>
-        <sz val="9.00"/>
-        <color rgb="FF1A1A1A"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">Avance como decimal entre 0 y 1. La barra verde crece automáticamente.
@@ -497,9 +500,9 @@
     </r>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
-        <sz val="11.00"/>
-        <color rgb="FF000000"/>
         <family val="2"/>
       </rPr>
       <t>Ejemplo: escriba 0.75 para representar el 75%.</t>
@@ -511,9 +514,9 @@
   <si>
     <r>
       <rPr>
+        <sz val="9"/>
+        <color rgb="FF1A1A1A"/>
         <rFont val="Arial"/>
-        <sz val="9.00"/>
-        <color rgb="FF1A1A1A"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">Estado actual de la actividad. Menú desplegable.
@@ -521,9 +524,9 @@
     </r>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
-        <sz val="11.00"/>
-        <color rgb="FF000000"/>
         <family val="2"/>
       </rPr>
       <t>El color se asigna automáticamente.</t>
@@ -532,10 +535,10 @@
   <si>
     <r>
       <rPr>
+        <i/>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
         <rFont val="Arial"/>
-        <sz val="9.00"/>
-        <i/>
-        <color rgb="FF666666"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">✅ Completado · ⏳ En proceso
@@ -543,14 +546,21 @@
     </r>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
-        <sz val="11.00"/>
-        <color rgb="FF000000"/>
         <family val="2"/>
       </rPr>
       <t>📅 Pendiente · 🔴 Crític</t>
     </r>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>o</t>
     </r>
   </si>
@@ -595,111 +605,177 @@
   </si>
   <si>
     <t>🎓  Raúl Bareño Gutiérrez  (Líder / Docente)</t>
+  </si>
+  <si>
+    <t>HU 11: Diseño y Creación de la Base de Datos Relacional (MySQL)</t>
+  </si>
+  <si>
+    <t>HU 13: Configuración de Infraestructura de Datos (Docker)</t>
+  </si>
+  <si>
+    <t>HU 14: Arquitectura Base y Monorepo</t>
+  </si>
+  <si>
+    <t>media</t>
+  </si>
+  <si>
+    <t>queda pendiente para revisar por Juan Diego para revisar si esta completa</t>
+  </si>
+  <si>
+    <t>Equipo: Sebastián Bautista Martínez, María Virginia Labarca, Andres Felipe Andrade</t>
+  </si>
+  <si>
+    <t>HU 15: Clasificación de Dataset de Caos para Entrenamiento de IA</t>
+  </si>
+  <si>
+    <t>Equipo: Pohlman Cuartas y  Oscar Antury Avila</t>
+  </si>
+  <si>
+    <t>El Equipo no entrego la tarea, y se reasigna a Juan Diego para completar esta HU</t>
+  </si>
+  <si>
+    <t>base de datos</t>
+  </si>
+  <si>
+    <t>infraestructura</t>
+  </si>
+  <si>
+    <t>datasets</t>
+  </si>
+  <si>
+    <t>Entregable 3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14">
+  <numFmts count="3">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color rgb="FF1A1A1A"/>
       <name val="Arial"/>
-      <sz val="9.00"/>
-      <color rgb="FF1A1A1A"/>
       <family val="2"/>
     </font>
     <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <sz val="12.00"/>
-      <b/>
-      <color rgb="FFFFFFFF"/>
       <family val="2"/>
     </font>
     <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF666666"/>
       <name val="Arial"/>
-      <sz val="9.00"/>
-      <u val="single"/>
-      <color rgb="FF1A1A1A"/>
       <family val="2"/>
     </font>
     <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <sz val="9.00"/>
-      <i/>
-      <color rgb="FF666666"/>
       <family val="2"/>
     </font>
     <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF5A8500"/>
       <name val="Arial"/>
-      <sz val="10.00"/>
-      <b/>
-      <color rgb="FFFFFFFF"/>
       <family val="2"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <sz val="9.00"/>
-      <b/>
-      <color rgb="FF5A8500"/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0563C1"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <sz val="11.00"/>
-      <u val="single"/>
-      <color rgb="FF0563C1"/>
       <family val="2"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <sz val="11.00"/>
-      <u val="single"/>
-      <color rgb="FF000000"/>
       <family val="2"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <sz val="11.00"/>
-      <color rgb="FF000000"/>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <sz val="8.00"/>
-      <b/>
-      <color rgb="FFFFFFFF"/>
       <family val="2"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="0"/>
       <name val="Arial"/>
-      <sz val="9.00"/>
-      <b/>
-      <color rgb="FFFFFFFF"/>
       <family val="2"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <sz val="22.00"/>
-      <b/>
-      <color rgb="FFFFFFFF"/>
+      <u/>
+      <sz val="11"/>
+      <color theme="11"/>
+      <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="9.00"/>
-      <i/>
-      <color rgb="FF5A8500"/>
-      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="22">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -732,19 +808,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF5A8500"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -792,19 +856,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF80BC00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEDF7D6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -826,8 +878,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="18">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -896,6 +954,126 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color rgb="FF80BC00"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF80BC00"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF80BC00"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF80BC00"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB8DC6E"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB8DC6E"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF80BC00"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF80BC00"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFCCCCCC"/>
       </left>
@@ -940,277 +1118,147 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB8DC6E"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB8DC6E"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF80BC00"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF80BC00"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF80BC00"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF80BC00"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF80BC00"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF80BC00"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF80BC00"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF80BC00"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF80BC00"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF80BC00"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="23">
+  <cellStyleXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf fontId="1" applyFont="1" fillId="2" applyFill="1" borderId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf fontId="2" applyFont="1" fillId="3" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf fontId="1" applyFont="1" fillId="4" applyFill="1" borderId="3" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf fontId="3" applyFont="1" fillId="5" applyFill="1" borderId="4" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf fontId="4" applyFont="1" fillId="6" applyFill="1" borderId="5" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf fontId="5" applyFont="1" fillId="7" applyFill="1" borderId="6" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf fontId="6" applyFont="1" fillId="8" applyFill="1" borderId="7" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf fontId="7" applyFont="1" fillId="9" applyFill="1" borderId="8" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf fontId="8" applyFont="1"/>
-    <xf fontId="6" applyFont="1" fillId="10" applyFill="1" borderId="9" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf fontId="9" applyFont="1" fillId="11" applyFill="1"/>
-    <xf fontId="10" applyFont="1" fillId="12" applyFill="1" borderId="10" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf fontId="9" applyFont="1" fillId="13" applyFill="1"/>
-    <xf fontId="10" applyFont="1" fillId="14" applyFill="1" borderId="11" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf fontId="11" applyFont="1" fillId="15" applyFill="1" borderId="12" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf fontId="12" applyFont="1" fillId="16" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf fontId="1" applyFont="1" fillId="17" applyFill="1" borderId="13" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf fontId="13" applyFont="1" fillId="18" applyFill="1" borderId="14" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf fontId="4" applyFont="1" fillId="19" applyFill="1" borderId="15" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf fontId="9" applyFont="1" fillId="20" applyFill="1" borderId="16" applyBorder="1"/>
-    <xf fontId="1" applyFont="1" fillId="21" applyFill="1" borderId="17" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf fontId="9" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf xfId="11" quotePrefix="0" pivotButton="0" fontId="9" applyFont="1" fillId="11" applyFill="1"/>
-    <xf xfId="16" quotePrefix="0" pivotButton="0" fontId="12" applyFont="1" fillId="16" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf xfId="8" quotePrefix="0" pivotButton="0" fontId="7" applyFont="1" fillId="9" applyFill="1" borderId="8" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="5" quotePrefix="0" pivotButton="0" fontId="4" applyFont="1" fillId="6" applyFill="1" borderId="5" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="7" quotePrefix="0" pivotButton="0" fontId="6" applyFont="1" fillId="8" applyFill="1" borderId="7" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="19" quotePrefix="0" pivotButton="0" fontId="4" applyFont="1" fillId="19" applyFill="1" borderId="15" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="10" quotePrefix="0" pivotButton="0" fontId="6" applyFont="1" fillId="10" applyFill="1" borderId="9" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="14" quotePrefix="0" pivotButton="0" fontId="10" applyFont="1" fillId="14" applyFill="1" borderId="11" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf xfId="22" quotePrefix="0" pivotButton="0" fontId="9" applyFont="1"/>
-    <xf xfId="12" quotePrefix="0" pivotButton="0" fontId="10" applyFont="1" fillId="12" applyFill="1" borderId="10" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left"/>
-    </xf>
-    <xf xfId="21" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="21" applyFill="1" borderId="17" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="13" quotePrefix="0" pivotButton="0" fontId="9" applyFont="1" fillId="13" applyFill="1"/>
-    <xf xfId="15" quotePrefix="0" pivotButton="0" fontId="11" applyFont="1" fillId="15" applyFill="1" borderId="12" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="17" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="17" applyFill="1" borderId="13" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="3" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="4" applyFill="1" borderId="3" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="1" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="2" applyFill="1" borderId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="9" quotePrefix="0" pivotButton="0" fontId="8" applyFont="1"/>
-    <xf xfId="4" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1" fillId="5" applyFill="1" borderId="4" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="2" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" fillId="3" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf xfId="20" quotePrefix="0" pivotButton="0" fontId="9" applyFont="1" fillId="20" applyFill="1" borderId="16" applyBorder="1"/>
-    <xf xfId="6" quotePrefix="0" pivotButton="0" fontId="5" applyFont="1" fillId="7" applyFill="1" borderId="6" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf xfId="18" quotePrefix="0" pivotButton="0" fontId="13" applyFont="1" fillId="18" applyFill="1" borderId="14" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="14" xfId="16" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="14" xfId="16" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="13" xfId="15" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="8" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="10" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="18" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="9" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="15" xfId="17" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="11" xfId="13" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="12" xfId="14" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="18" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="18" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="18" borderId="15" xfId="17" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="13" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="14" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="17" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="19"/>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="15" xfId="17" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="9" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="18" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="10" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="normal" xfId="0" builtinId="0"/>
+  <cellStyles count="8">
+    <cellStyle name="Hipervínculo" xfId="19" builtinId="8"/>
+    <cellStyle name="Hipervínculo visitado" xfId="10" builtinId="9"/>
+    <cellStyle name="Millares" xfId="5" builtinId="3"/>
+    <cellStyle name="Millares [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Moneda [0]" xfId="3" builtinId="7"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentaje" xfId="2" builtinId="5"/>
+    <cellStyle name="Título" xfId="1" builtinId="15"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1487,194 +1535,198 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.00" customHeight="1" defaultColWidth="8.71"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:O33"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.43" customWidth="1" hidden="0"/>
-    <col min="2" max="2" width="13.37" customWidth="1" hidden="0"/>
-    <col min="3" max="3" width="54.58" customWidth="1" hidden="0"/>
-    <col min="4" max="4" width="32.13" customWidth="1" hidden="0"/>
-    <col min="5" max="5" width="11.28" customWidth="1" hidden="0"/>
-    <col min="6" max="6" width="50.04" customWidth="1" hidden="0"/>
-    <col min="7" max="7" width="14.23" customWidth="1" hidden="0"/>
-    <col min="8" max="9" width="10.67" customWidth="1" hidden="0"/>
-    <col min="10" max="10" width="17.54" customWidth="1" hidden="0"/>
-    <col min="11" max="11" width="10.67" customWidth="1" hidden="0"/>
-    <col min="12" max="12" width="10.18" customWidth="1" hidden="0"/>
-    <col min="13" max="13" width="14.72" customWidth="1" hidden="0"/>
-    <col min="14" max="14" width="18.40" customWidth="1" hidden="0"/>
-    <col min="15" max="15" width="32.75" customWidth="1" hidden="0"/>
+    <col min="1" max="1" width="10.42578125" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" customWidth="1"/>
+    <col min="3" max="3" width="54.5703125" customWidth="1"/>
+    <col min="4" max="4" width="32.140625" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" customWidth="1"/>
+    <col min="6" max="6" width="67.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" customWidth="1"/>
+    <col min="8" max="9" width="10.7109375" customWidth="1"/>
+    <col min="10" max="10" width="17.5703125" customWidth="1"/>
+    <col min="11" max="11" width="10.7109375" customWidth="1"/>
+    <col min="12" max="12" width="10.140625" customWidth="1"/>
+    <col min="13" max="13" width="14.7109375" customWidth="1"/>
+    <col min="14" max="14" width="18.42578125" customWidth="1"/>
+    <col min="15" max="15" width="66.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.00" customHeight="true">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-    </row>
-    <row r="2" ht="15.00" customHeight="true">
-      <c r="A2" s="2" t="s">
+    <row r="1" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="3"/>
+      <c r="O1" s="3"/>
+    </row>
+    <row r="2" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="4" t="s">
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-    </row>
-    <row r="3" ht="15.00" customHeight="true">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="5" t="s">
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="14"/>
+    </row>
+    <row r="3" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="15"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
-    </row>
-    <row r="4" ht="15.00" customHeight="true">
-      <c r="A4" s="2"/>
-      <c r="B4" s="6" t="s">
+      <c r="L3" s="13"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="13"/>
+      <c r="O3" s="13"/>
+    </row>
+    <row r="4" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="15"/>
+      <c r="B4" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="7" t="s">
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="L4" s="7"/>
-      <c r="M4" s="7"/>
-      <c r="N4" s="7"/>
-      <c r="O4" s="7"/>
-    </row>
-    <row r="5" ht="15.00" customHeight="true">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-    </row>
-    <row r="6" ht="15.00" customHeight="true">
+      <c r="L4" s="11"/>
+      <c r="M4" s="11"/>
+      <c r="N4" s="11"/>
+      <c r="O4" s="11"/>
+    </row>
+    <row r="5" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+    </row>
+    <row r="6" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
       <c r="F6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
       <c r="J6" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="K6" s="9" t="s">
+      <c r="K6" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="9"/>
+      <c r="L6" s="17"/>
       <c r="M6" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="N6" s="9" t="s">
+      <c r="N6" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="O6" s="9"/>
-    </row>
-    <row r="7" ht="15.00" customHeight="true">
+      <c r="O6" s="17"/>
+    </row>
+    <row r="7" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="11"/>
+      <c r="C7" s="16"/>
       <c r="D7" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="11"/>
+      <c r="F7" s="16"/>
       <c r="G7" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="11" t="s">
+      <c r="H7" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="I7" s="11"/>
+      <c r="I7" s="16"/>
       <c r="J7" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="K7" s="11">
-        <f>=COUNTA(A10:A32)</f>
-      </c>
-      <c r="L7" s="11"/>
+      <c r="K7" s="16">
+        <f>COUNTA(A10:A32)</f>
+        <v>18</v>
+      </c>
+      <c r="L7" s="16"/>
       <c r="M7" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="N7" s="11">
-        <f>=COUNTIF(M10:M32,"✅ Completado")</f>
-      </c>
-      <c r="O7" s="11"/>
-    </row>
-    <row r="8" ht="15.00" customHeight="true">
+      <c r="N7" s="16">
+        <f>COUNTIF(M10:M32,"✅ Completado")</f>
+        <v>22</v>
+      </c>
+      <c r="O7" s="16"/>
+    </row>
+    <row r="8" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="12"/>
       <c r="B8" s="12"/>
       <c r="C8" s="12"/>
@@ -1691,7 +1743,7 @@
       <c r="N8" s="12"/>
       <c r="O8" s="12"/>
     </row>
-    <row r="9" ht="39.00" customHeight="true">
+    <row r="9" spans="1:15" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
         <v>22</v>
       </c>
@@ -1738,921 +1790,1029 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" ht="15.00" customHeight="true">
+    <row r="10" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11">
         <v>1</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="26">
         <v>3</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="H10" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="I10" s="9" t="s">
+      <c r="I10" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="11" t="s">
+      <c r="J10" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="K10" s="11" t="s">
+      <c r="K10" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="L10" s="11">
+      <c r="L10" s="26">
         <v>1</v>
       </c>
-      <c r="M10" s="11" t="s">
+      <c r="M10" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="N10" s="11" t="s">
+      <c r="N10" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="O10" s="14" t="s">
+      <c r="O10" s="24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="11" ht="15.00" customHeight="true">
+    <row r="11" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="15">
         <v>2</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="26">
         <v>3</v>
       </c>
-      <c r="F11" s="16" t="s">
+      <c r="F11" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="H11" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="I11" s="9" t="s">
+      <c r="I11" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="J11" s="15" t="s">
+      <c r="J11" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="K11" s="11" t="s">
+      <c r="K11" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="L11" s="11">
+      <c r="L11" s="26">
         <v>1</v>
       </c>
-      <c r="M11" s="11" t="s">
+      <c r="M11" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="N11" s="11" t="s">
+      <c r="N11" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="O11" s="14" t="s">
+      <c r="O11" s="24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="12" ht="15.00" customHeight="true">
+    <row r="12" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11">
         <v>3</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="E12" s="11">
+      <c r="E12" s="26">
         <v>3</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="F12" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="H12" s="9" t="s">
+      <c r="H12" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="I12" s="9" t="s">
+      <c r="I12" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="J12" s="11" t="s">
+      <c r="J12" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="K12" s="11" t="s">
+      <c r="K12" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="L12" s="11">
+      <c r="L12" s="26">
         <v>1</v>
       </c>
-      <c r="M12" s="11" t="s">
+      <c r="M12" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="N12" s="11" t="s">
+      <c r="N12" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="O12" s="14" t="s">
+      <c r="O12" s="24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="13" ht="15.00" customHeight="true">
+    <row r="13" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="15">
         <v>4</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="26">
         <v>3</v>
       </c>
-      <c r="F13" s="16" t="s">
+      <c r="F13" s="28" t="s">
         <v>53</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="H13" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="I13" s="9" t="s">
+      <c r="I13" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="11" t="s">
+      <c r="J13" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="K13" s="11" t="s">
+      <c r="K13" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="L13" s="11">
+      <c r="L13" s="26">
         <v>1</v>
       </c>
-      <c r="M13" s="11" t="s">
+      <c r="M13" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="N13" s="11" t="s">
+      <c r="N13" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="O13" s="14" t="s">
+      <c r="O13" s="24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="14" ht="15.00" customHeight="true">
+    <row r="14" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11">
         <v>5</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="26">
         <v>3</v>
       </c>
-      <c r="F14" s="14" t="s">
+      <c r="F14" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="H14" s="9" t="s">
+      <c r="H14" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="I14" s="9" t="s">
+      <c r="I14" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="J14" s="15" t="s">
+      <c r="J14" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="K14" s="11" t="s">
+      <c r="K14" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="L14" s="11">
+      <c r="L14" s="26">
         <v>1</v>
       </c>
-      <c r="M14" s="11" t="s">
+      <c r="M14" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="N14" s="11" t="s">
+      <c r="N14" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="O14" s="14" t="s">
+      <c r="O14" s="24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="15" ht="15.00" customHeight="true">
+    <row r="15" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="15">
         <v>6</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="E15" s="11">
+      <c r="E15" s="26">
         <v>3</v>
       </c>
-      <c r="F15" s="16" t="s">
+      <c r="F15" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="H15" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="I15" s="9" t="s">
+      <c r="I15" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="J15" s="11" t="s">
+      <c r="J15" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="K15" s="11" t="s">
+      <c r="K15" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="L15" s="11">
+      <c r="L15" s="26">
         <v>1</v>
       </c>
-      <c r="M15" s="11" t="s">
+      <c r="M15" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="N15" s="11" t="s">
+      <c r="N15" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="O15" s="14" t="s">
+      <c r="O15" s="24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="16" ht="15.00" customHeight="true">
+    <row r="16" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11">
         <v>7</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="C16" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="26">
         <v>3</v>
       </c>
-      <c r="F16" s="14" t="s">
+      <c r="F16" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="H16" s="9" t="s">
+      <c r="H16" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="I16" s="9" t="s">
+      <c r="I16" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="J16" s="11" t="s">
+      <c r="J16" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="K16" s="11" t="s">
+      <c r="K16" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="L16" s="11">
+      <c r="L16" s="26">
         <v>1</v>
       </c>
-      <c r="M16" s="11" t="s">
+      <c r="M16" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="N16" s="11" t="s">
+      <c r="N16" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="O16" s="14" t="s">
+      <c r="O16" s="24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="17" ht="15.00" customHeight="true">
+    <row r="17" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="15">
         <v>10</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="C17" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="E17" s="11">
+      <c r="E17" s="26">
         <v>3</v>
       </c>
-      <c r="F17" s="16" t="s">
+      <c r="F17" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="H17" s="9" t="s">
+      <c r="H17" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="I17" s="9" t="s">
+      <c r="I17" s="27" t="s">
         <v>65</v>
       </c>
-      <c r="J17" s="11" t="s">
+      <c r="J17" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="K17" s="11" t="s">
+      <c r="K17" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="L17" s="11">
+      <c r="L17" s="26">
         <v>1</v>
       </c>
-      <c r="M17" s="11" t="s">
+      <c r="M17" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="N17" s="11" t="s">
+      <c r="N17" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="O17" s="14" t="s">
+      <c r="O17" s="24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="18" ht="15.00" customHeight="true">
+    <row r="18" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
         <v>11</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="E18" s="11">
+      <c r="E18" s="26">
         <v>3</v>
       </c>
-      <c r="F18" s="14" t="s">
+      <c r="F18" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="G18" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="H18" s="9" t="s">
+      <c r="H18" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="I18" s="9" t="s">
+      <c r="I18" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="J18" s="15" t="s">
+      <c r="J18" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="K18" s="11" t="s">
+      <c r="K18" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="L18" s="11">
+      <c r="L18" s="26">
         <v>1</v>
       </c>
-      <c r="M18" s="11" t="s">
+      <c r="M18" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="N18" s="11" t="s">
+      <c r="N18" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="O18" s="14" t="s">
+      <c r="O18" s="24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="19" ht="15.00" customHeight="true">
+    <row r="19" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="15">
         <v>12</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="28" t="s">
         <v>68</v>
       </c>
-      <c r="C19" s="16" t="s">
+      <c r="C19" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="E19" s="11">
+      <c r="E19" s="26">
         <v>3</v>
       </c>
-      <c r="F19" s="16" t="s">
+      <c r="F19" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="G19" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="H19" s="9" t="s">
+      <c r="H19" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="I19" s="9" t="s">
+      <c r="I19" s="27" t="s">
         <v>71</v>
       </c>
-      <c r="J19" s="11" t="s">
+      <c r="J19" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="K19" s="11" t="s">
+      <c r="K19" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="L19" s="11">
+      <c r="L19" s="26">
         <v>1</v>
       </c>
-      <c r="M19" s="11" t="s">
+      <c r="M19" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="N19" s="11" t="s">
+      <c r="N19" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="O19" s="14" t="s">
+      <c r="O19" s="24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="20" ht="15.00" customHeight="true">
+    <row r="20" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11">
         <v>13</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="C20" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="E20" s="11">
+      <c r="E20" s="26">
         <v>3</v>
       </c>
-      <c r="F20" s="14" t="s">
+      <c r="F20" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="G20" s="9" t="s">
+      <c r="G20" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="H20" s="9" t="s">
+      <c r="H20" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="I20" s="9" t="s">
+      <c r="I20" s="27" t="s">
         <v>75</v>
       </c>
-      <c r="J20" s="11" t="s">
+      <c r="J20" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="K20" s="11" t="s">
+      <c r="K20" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="L20" s="11">
+      <c r="L20" s="26">
         <v>1</v>
       </c>
-      <c r="M20" s="11" t="s">
+      <c r="M20" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="N20" s="11" t="s">
+      <c r="N20" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="O20" s="14" t="s">
+      <c r="O20" s="24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="21" ht="15.00" customHeight="true">
+    <row r="21" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="15">
         <v>14</v>
       </c>
-      <c r="B21" s="16" t="s">
+      <c r="B21" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="C21" s="16" t="s">
+      <c r="C21" s="28" t="s">
         <v>77</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="E21" s="11">
+      <c r="E21" s="26">
         <v>3</v>
       </c>
-      <c r="F21" s="16" t="s">
+      <c r="F21" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="G21" s="9" t="s">
+      <c r="G21" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="H21" s="9" t="s">
+      <c r="H21" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="I21" s="9" t="s">
+      <c r="I21" s="27" t="s">
         <v>78</v>
       </c>
-      <c r="J21" s="15" t="s">
+      <c r="J21" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="K21" s="11" t="s">
+      <c r="K21" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="L21" s="11">
+      <c r="L21" s="26">
         <v>1</v>
       </c>
-      <c r="M21" s="15" t="s">
+      <c r="M21" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="N21" s="11" t="s">
+      <c r="N21" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="O21" s="14" t="s">
+      <c r="O21" s="24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="22" ht="15.00" customHeight="true">
+    <row r="22" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11">
         <v>15</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="B22" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="C22" s="14" t="s">
+      <c r="C22" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="E22" s="11">
+      <c r="E22" s="26">
         <v>3</v>
       </c>
-      <c r="F22" s="14" t="s">
+      <c r="F22" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="G22" s="9" t="s">
+      <c r="G22" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="H22" s="9" t="s">
+      <c r="H22" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="I22" s="9" t="s">
+      <c r="I22" s="27" t="s">
         <v>80</v>
       </c>
-      <c r="J22" s="11" t="s">
+      <c r="J22" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="K22" s="11" t="s">
+      <c r="K22" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="L22" s="11">
+      <c r="L22" s="26">
         <v>1</v>
       </c>
-      <c r="M22" s="11" t="s">
+      <c r="M22" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="N22" s="11" t="s">
+      <c r="N22" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="O22" s="14" t="s">
+      <c r="O22" s="24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="23" ht="15.00" customHeight="true">
+    <row r="23" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="15">
         <v>16</v>
       </c>
-      <c r="B23" s="16" t="s">
+      <c r="B23" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="C23" s="16" t="s">
+      <c r="C23" s="28" t="s">
         <v>81</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="E23" s="11">
+      <c r="E23" s="26">
         <v>3</v>
       </c>
-      <c r="F23" s="16" t="s">
+      <c r="F23" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="G23" s="9" t="s">
+      <c r="G23" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="H23" s="9" t="s">
+      <c r="H23" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="I23" s="9" t="s">
+      <c r="I23" s="27" t="s">
         <v>82</v>
       </c>
-      <c r="J23" s="11" t="s">
+      <c r="J23" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="K23" s="11" t="s">
+      <c r="K23" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="L23" s="11">
+      <c r="L23" s="26">
         <v>1</v>
       </c>
-      <c r="M23" s="15" t="s">
+      <c r="M23" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="N23" s="11" t="s">
+      <c r="N23" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="O23" s="14" t="s">
+      <c r="O23" s="24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="24" ht="15.00" customHeight="true">
+    <row r="24" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11">
         <v>17</v>
       </c>
-      <c r="B24" s="14" t="s">
+      <c r="B24" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="C24" s="14" t="s">
+      <c r="C24" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="E24" s="11">
+      <c r="E24" s="26">
         <v>3</v>
       </c>
-      <c r="F24" s="14" t="s">
+      <c r="F24" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="G24" s="17" t="s">
+      <c r="G24" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="H24" s="9" t="s">
+      <c r="H24" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="I24" s="9" t="s">
+      <c r="I24" s="27" t="s">
         <v>84</v>
       </c>
-      <c r="J24" s="15" t="s">
+      <c r="J24" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="K24" s="11" t="s">
+      <c r="K24" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="L24" s="11">
+      <c r="L24" s="26">
         <v>1</v>
       </c>
-      <c r="M24" s="11" t="s">
+      <c r="M24" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="N24" s="11" t="s">
+      <c r="N24" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="O24" s="14" t="s">
+      <c r="O24" s="24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="25" ht="15.00" customHeight="true">
+    <row r="25" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="15">
         <v>18</v>
       </c>
-      <c r="B25" s="16" t="s">
+      <c r="B25" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="C25" s="16" t="s">
+      <c r="C25" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D25" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="E25" s="11">
+      <c r="E25" s="26">
         <v>3</v>
       </c>
-      <c r="F25" s="16" t="s">
+      <c r="F25" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="G25" s="9" t="s">
+      <c r="G25" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="H25" s="9" t="s">
+      <c r="H25" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="I25" s="9" t="s">
+      <c r="I25" s="27" t="s">
         <v>87</v>
       </c>
-      <c r="J25" s="11" t="s">
+      <c r="J25" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="K25" s="11" t="s">
+      <c r="K25" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="L25" s="11">
+      <c r="L25" s="26">
         <v>1</v>
       </c>
-      <c r="M25" s="15" t="s">
+      <c r="M25" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="N25" s="11" t="s">
+      <c r="N25" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="O25" s="14" t="s">
+      <c r="O25" s="24" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="26" ht="15.00" customHeight="true">
+    <row r="26" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11">
         <v>19</v>
       </c>
-      <c r="B26" s="14" t="s">
+      <c r="B26" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="C26" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="E26" s="11">
+      <c r="E26" s="26">
         <v>3</v>
       </c>
-      <c r="F26" s="14" t="s">
+      <c r="F26" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="G26" s="9" t="s">
+      <c r="G26" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="H26" s="9" t="s">
+      <c r="H26" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="I26" s="9" t="s">
+      <c r="I26" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="J26" s="11" t="s">
+      <c r="J26" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="K26" s="11" t="s">
+      <c r="K26" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="L26" s="11">
+      <c r="L26" s="26">
         <v>1</v>
       </c>
-      <c r="M26" s="11" t="s">
+      <c r="M26" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="N26" s="11" t="s">
+      <c r="N26" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="O26" s="14" t="s">
+      <c r="O26" s="24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="27" ht="15.00" customHeight="true">
+    <row r="27" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="15">
         <v>20</v>
       </c>
-      <c r="B27" s="16" t="s">
+      <c r="B27" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="C27" s="16" t="s">
+      <c r="C27" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="E27" s="11">
+      <c r="E27" s="26">
         <v>3</v>
       </c>
-      <c r="F27" s="16" t="s">
+      <c r="F27" s="28" t="s">
         <v>93</v>
       </c>
-      <c r="G27" s="9" t="s">
+      <c r="G27" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="H27" s="9" t="s">
+      <c r="H27" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="I27" s="9" t="s">
+      <c r="I27" s="27" t="s">
         <v>94</v>
       </c>
-      <c r="J27" s="15" t="s">
+      <c r="J27" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="K27" s="11" t="s">
+      <c r="K27" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="L27" s="15">
+      <c r="L27" s="29">
         <v>1</v>
       </c>
-      <c r="M27" s="15" t="s">
+      <c r="M27" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="N27" s="11" t="s">
+      <c r="N27" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="O27" s="14" t="s">
+      <c r="O27" s="24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="28" ht="15.00" customHeight="true">
+    <row r="28" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="11"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="11"/>
-      <c r="H28" s="11"/>
-      <c r="I28" s="11"/>
-      <c r="J28" s="11"/>
-      <c r="K28" s="11"/>
-      <c r="L28" s="11"/>
-      <c r="M28" s="18"/>
-      <c r="N28" s="11"/>
-      <c r="O28" s="14"/>
-    </row>
-    <row r="29" ht="15.00" customHeight="true">
+      <c r="B28" s="24" t="s">
+        <v>151</v>
+      </c>
+      <c r="C28" s="24" t="s">
+        <v>142</v>
+      </c>
+      <c r="D28" s="30" t="s">
+        <v>154</v>
+      </c>
+      <c r="E28" s="26">
+        <v>3</v>
+      </c>
+      <c r="F28" s="24" t="s">
+        <v>147</v>
+      </c>
+      <c r="G28" s="27">
+        <v>46086</v>
+      </c>
+      <c r="H28" s="27">
+        <v>46270</v>
+      </c>
+      <c r="I28" s="27">
+        <v>46271</v>
+      </c>
+      <c r="J28" s="26" t="s">
+        <v>145</v>
+      </c>
+      <c r="K28" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="L28" s="26">
+        <v>1</v>
+      </c>
+      <c r="M28" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="N28" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="O28" s="24" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="15"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="15"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="15"/>
-      <c r="H29" s="15"/>
-      <c r="I29" s="15"/>
-      <c r="J29" s="15"/>
-      <c r="K29" s="15"/>
-      <c r="L29" s="15"/>
-      <c r="M29" s="15"/>
-      <c r="N29" s="15"/>
-      <c r="O29" s="16"/>
-    </row>
-    <row r="30" ht="15.00" customHeight="true">
+      <c r="B29" s="28" t="s">
+        <v>152</v>
+      </c>
+      <c r="C29" s="28" t="s">
+        <v>143</v>
+      </c>
+      <c r="D29" s="30" t="s">
+        <v>154</v>
+      </c>
+      <c r="E29" s="26">
+        <v>3</v>
+      </c>
+      <c r="F29" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="G29" s="27">
+        <v>46086</v>
+      </c>
+      <c r="H29" s="27">
+        <v>46270</v>
+      </c>
+      <c r="I29" s="27">
+        <v>46271</v>
+      </c>
+      <c r="J29" s="26" t="s">
+        <v>145</v>
+      </c>
+      <c r="K29" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="L29" s="26">
+        <v>1</v>
+      </c>
+      <c r="M29" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="N29" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="O29" s="24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="11"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="11"/>
-      <c r="H30" s="11"/>
-      <c r="I30" s="11"/>
-      <c r="J30" s="11"/>
-      <c r="K30" s="11"/>
-      <c r="L30" s="11"/>
-      <c r="M30" s="11"/>
-      <c r="N30" s="11"/>
-      <c r="O30" s="14"/>
-    </row>
-    <row r="31" ht="15.00" customHeight="true">
-      <c r="A31" s="15"/>
-      <c r="B31" s="16"/>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="15"/>
-      <c r="F31" s="16"/>
-      <c r="G31" s="15"/>
-      <c r="H31" s="15"/>
-      <c r="I31" s="15"/>
-      <c r="J31" s="15"/>
-      <c r="K31" s="15"/>
-      <c r="L31" s="15"/>
-      <c r="M31" s="15"/>
-      <c r="N31" s="15"/>
-      <c r="O31" s="16"/>
-    </row>
-    <row r="32" ht="15.00" customHeight="true">
+      <c r="B30" s="28" t="s">
+        <v>152</v>
+      </c>
+      <c r="C30" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="D30" s="30" t="s">
+        <v>154</v>
+      </c>
+      <c r="E30" s="26">
+        <v>3</v>
+      </c>
+      <c r="F30" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="G30" s="27">
+        <v>46086</v>
+      </c>
+      <c r="H30" s="27">
+        <v>46270</v>
+      </c>
+      <c r="I30" s="27">
+        <v>46271</v>
+      </c>
+      <c r="J30" s="26" t="s">
+        <v>145</v>
+      </c>
+      <c r="K30" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="L30" s="29">
+        <v>1</v>
+      </c>
+      <c r="M30" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="N30" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="O30" s="24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" s="23" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="19"/>
+      <c r="B31" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="C31" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="D31" s="20"/>
+      <c r="E31" s="21">
+        <v>3</v>
+      </c>
+      <c r="F31" s="20" t="s">
+        <v>149</v>
+      </c>
+      <c r="G31" s="22">
+        <v>46086</v>
+      </c>
+      <c r="H31" s="22">
+        <v>46270</v>
+      </c>
+      <c r="I31" s="22"/>
+      <c r="J31" s="21" t="s">
+        <v>145</v>
+      </c>
+      <c r="K31" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="L31" s="21">
+        <v>1</v>
+      </c>
+      <c r="M31" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="N31" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="O31" s="20" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="11"/>
       <c r="B32" s="14"/>
       <c r="C32" s="14"/>
@@ -2669,26 +2829,27 @@
       <c r="N32" s="11"/>
       <c r="O32" s="14"/>
     </row>
-    <row r="33" ht="15.75" customHeight="true">
-      <c r="A33" s="17" t="s">
+    <row r="33" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="B33" s="17"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
-      <c r="G33" s="17"/>
-      <c r="H33" s="17"/>
-      <c r="I33" s="17"/>
-      <c r="J33" s="17"/>
-      <c r="K33" s="17"/>
-      <c r="L33" s="19">
-        <f>=IFERROR(AVERAGEIF(L10:L32,"&gt;0",L10:L32),0)</f>
-      </c>
-      <c r="M33" s="20"/>
-      <c r="N33" s="20"/>
-      <c r="O33" s="20"/>
+      <c r="B33" s="18"/>
+      <c r="C33" s="18"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="18"/>
+      <c r="G33" s="18"/>
+      <c r="H33" s="18"/>
+      <c r="I33" s="18"/>
+      <c r="J33" s="18"/>
+      <c r="K33" s="18"/>
+      <c r="L33" s="17">
+        <f>IFERROR(AVERAGEIF(L10:L32,"&gt;0",L10:L32),0)</f>
+        <v>1</v>
+      </c>
+      <c r="M33" s="2"/>
+      <c r="N33" s="2"/>
+      <c r="O33" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -2710,59 +2871,62 @@
     <mergeCell ref="N7:O7"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D28" r:id="rId1" tooltip="Entregable 3" display="https://github.com/IA-DataFlow-Hub/docs/tree/main/Requisitos para aprobar el semillero/6 - Entregas Parciales/Entregable 3" xr:uid="{717E635B-02DC-4654-858B-0C3CF6195584}"/>
+    <hyperlink ref="D29" r:id="rId2" tooltip="Entregable 3" display="https://github.com/IA-DataFlow-Hub/docs/tree/main/Requisitos para aprobar el semillero/6 - Entregas Parciales/Entregable 3" xr:uid="{5CA9E379-F4E5-4322-890C-EB26CFA0D350}"/>
+    <hyperlink ref="D30" r:id="rId3" tooltip="Entregable 3" display="https://github.com/IA-DataFlow-Hub/docs/tree/main/Requisitos para aprobar el semillero/6 - Entregas Parciales/Entregable 3" xr:uid="{3F97DE31-EE13-4EDA-8237-EF249DA92A1B}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.75" header="0.25" footer="0.25"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100"/>
-  <headerFooter alignWithMargins="1"/>
+  <pageSetup paperSize="7" scale="31" fitToHeight="0" orientation="landscape" r:id="rId4"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.00" customHeight="1" defaultColWidth="8.71"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:A9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" ht="15.00" customHeight="true">
+    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="2" ht="15.00" customHeight="true">
+    <row r="2" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="3" ht="15.00" customHeight="true">
+    <row r="3" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="4" ht="15.00" customHeight="true">
+    <row r="4" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="5" ht="15.00" customHeight="true">
+    <row r="5" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="6" ht="15.00" customHeight="true">
+    <row r="6" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="7" ht="15.00" customHeight="true">
+    <row r="7" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="8" ht="15.00" customHeight="true">
+    <row r="8" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="9" ht="15.00" customHeight="true">
+    <row r="9" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>9</v>
       </c>
@@ -2770,73 +2934,71 @@
   </sheetData>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.75" header="0.25" footer="0.25"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100"/>
-  <headerFooter alignWithMargins="1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.00" customHeight="1" defaultColWidth="8.71"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:D32"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.05" customWidth="1" hidden="0"/>
-    <col min="2" max="2" width="24.04" customWidth="1" hidden="0"/>
-    <col min="3" max="3" width="56.05" customWidth="1" hidden="0"/>
-    <col min="4" max="4" width="32.01" customWidth="1" hidden="0"/>
+    <col min="1" max="1" width="4" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="56" customWidth="1"/>
+    <col min="4" max="4" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="9.75" customHeight="true">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-    </row>
-    <row r="2" ht="49.50" customHeight="true">
-      <c r="A2" s="16" t="s">
+    <row r="1" spans="1:4" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+    </row>
+    <row r="2" spans="1:4" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="32" t="s">
         <v>97</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-    </row>
-    <row r="3" ht="19.50" customHeight="true">
-      <c r="A3" s="16"/>
-      <c r="B3" s="6" t="s">
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+    </row>
+    <row r="3" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="31"/>
+      <c r="B3" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-    </row>
-    <row r="4" ht="18.00" customHeight="true">
-      <c r="A4" s="16"/>
-      <c r="B4" s="14" t="s">
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+    </row>
+    <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="31"/>
+      <c r="B4" s="33" t="s">
         <v>99</v>
       </c>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-    </row>
-    <row r="5" ht="4.50" customHeight="true">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-    </row>
-    <row r="7" ht="27.75" customHeight="true">
-      <c r="B7" s="21" t="s">
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+    </row>
+    <row r="5" spans="1:4" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+    </row>
+    <row r="7" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D7" s="21" t="s">
+      <c r="D7" s="18" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="8" ht="42.00" customHeight="true">
+    <row r="8" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="7" t="s">
         <v>22</v>
       </c>
@@ -2847,7 +3009,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="9" ht="42.00" customHeight="true">
+    <row r="9" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="5" t="s">
         <v>23</v>
       </c>
@@ -2858,7 +3020,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="10" ht="42.00" customHeight="true">
+    <row r="10" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="7" t="s">
         <v>24</v>
       </c>
@@ -2869,7 +3031,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="11" ht="42.00" customHeight="true">
+    <row r="11" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="5" t="s">
         <v>25</v>
       </c>
@@ -2880,7 +3042,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="12" ht="42.00" customHeight="true">
+    <row r="12" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="7" t="s">
         <v>111</v>
       </c>
@@ -2891,7 +3053,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="13" ht="42.00" customHeight="true">
+    <row r="13" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="5" t="s">
         <v>27</v>
       </c>
@@ -2902,7 +3064,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="14" ht="42.00" customHeight="true">
+    <row r="14" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="7" t="s">
         <v>116</v>
       </c>
@@ -2913,7 +3075,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="15" ht="42.00" customHeight="true">
+    <row r="15" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
         <v>31</v>
       </c>
@@ -2924,7 +3086,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="16" ht="42.00" customHeight="true">
+    <row r="16" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="7" t="s">
         <v>121</v>
       </c>
@@ -2935,7 +3097,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="17" ht="42.00" customHeight="true">
+    <row r="17" spans="2:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
         <v>33</v>
       </c>
@@ -2946,7 +3108,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="18" ht="42.00" customHeight="true">
+    <row r="18" spans="2:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="7" t="s">
         <v>34</v>
       </c>
@@ -2957,7 +3119,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="19" ht="42.00" customHeight="true">
+    <row r="19" spans="2:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="5" t="s">
         <v>128</v>
       </c>
@@ -2968,7 +3130,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="20" ht="42.00" customHeight="true">
+    <row r="20" spans="2:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="7" t="s">
         <v>36</v>
       </c>
@@ -2979,75 +3141,75 @@
         <v>108</v>
       </c>
     </row>
-    <row r="22" ht="45.75" customHeight="true">
-      <c r="B22" s="22" t="s">
+    <row r="22" spans="2:4" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="34" t="s">
         <v>132</v>
       </c>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-    </row>
-    <row r="24" ht="27.75" customHeight="true">
-      <c r="B24" s="21" t="s">
+      <c r="C22" s="34"/>
+      <c r="D22" s="34"/>
+    </row>
+    <row r="24" spans="2:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="C24" s="21"/>
-      <c r="D24" s="21"/>
-    </row>
-    <row r="25" ht="21.75" customHeight="true">
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+    </row>
+    <row r="25" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="9" t="s">
         <v>134</v>
       </c>
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
     </row>
-    <row r="26" ht="21.75" customHeight="true">
-      <c r="B26" s="20" t="s">
+    <row r="26" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
-    </row>
-    <row r="27" ht="21.75" customHeight="true">
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+    </row>
+    <row r="27" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="9" t="s">
         <v>136</v>
       </c>
       <c r="C27" s="9"/>
       <c r="D27" s="9"/>
     </row>
-    <row r="28" ht="21.75" customHeight="true">
-      <c r="B28" s="20" t="s">
+    <row r="28" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
-    </row>
-    <row r="29" ht="21.75" customHeight="true">
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+    </row>
+    <row r="29" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="9" t="s">
         <v>138</v>
       </c>
       <c r="C29" s="9"/>
       <c r="D29" s="9"/>
     </row>
-    <row r="30" ht="21.75" customHeight="true">
-      <c r="B30" s="20" t="s">
+    <row r="30" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
-    </row>
-    <row r="31" ht="21.75" customHeight="true">
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+    </row>
+    <row r="31" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="9" t="s">
         <v>140</v>
       </c>
       <c r="C31" s="9"/>
       <c r="D31" s="9"/>
     </row>
-    <row r="32" ht="21.75" customHeight="true">
-      <c r="B32" s="19" t="s">
+    <row r="32" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
+      <c r="C32" s="7"/>
+      <c r="D32" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -3068,7 +3230,6 @@
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.75" header="0.25" footer="0.25"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100"/>
-  <headerFooter alignWithMargins="1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-05-13 19:34:08
</commit_message>
<xml_diff>
--- a/Requisitos para aprobar el semillero/3 - Plan de Trabajo/Plan de trabajo FUAA.xlsx
+++ b/Requisitos para aprobar el semillero/3 - Plan de Trabajo/Plan de trabajo FUAA.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Areandina\Semillero\Docs\IA-DataFlow Hub - Semillero\Requisitos para aprobar el semillero\3 - Plan de Trabajo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mejia\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4BFDF2BC-2EF9-416D-894F-B055ED89C860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DBBC8AC-9F22-4D8D-9EB1-4B913CCE6F48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="201">
   <si>
     <t>A</t>
   </si>
@@ -645,6 +645,144 @@
   <si>
     <t>Entregable 3</t>
   </si>
+  <si>
+    <t>16/5/2026</t>
+  </si>
+  <si>
+    <t>Base de Datos</t>
+  </si>
+  <si>
+    <t>HU-016: Reemplazar ENUMs con Tablas de Catálogo</t>
+  </si>
+  <si>
+    <t>13/05/2026</t>
+  </si>
+  <si>
+    <t>19/05/2026</t>
+  </si>
+  <si>
+    <t>HU-017: Implementar Auditoría y Eliminación Lógica</t>
+  </si>
+  <si>
+    <t>HU-025: Sistema de Notificaciones Individuales y Grupales</t>
+  </si>
+  <si>
+    <t>Entregable 4</t>
+  </si>
+  <si>
+    <t>18/05/2026</t>
+  </si>
+  <si>
+    <t>25/05/2026</t>
+  </si>
+  <si>
+    <t>HU-026: Gestión de Datasets, Tablas y Lineage</t>
+  </si>
+  <si>
+    <t>HU-027: Gestión de Templates ETL y Transf. Predefinidas</t>
+  </si>
+  <si>
+    <t>HU-028: Feed de Actividad y Timeline de Eventos</t>
+  </si>
+  <si>
+    <t>HU-029: Sistema de Reportes y Dashboards Persistentes</t>
+  </si>
+  <si>
+    <t>HU-030: Migración Estratégica de IDs Enteros a UUID/GUID</t>
+  </si>
+  <si>
+    <t>Infraestructura</t>
+  </si>
+  <si>
+    <t>HU-035: Diagramas Clave del Proyecto</t>
+  </si>
+  <si>
+    <t>Equipo: Juan Diego Mejía y David Ospina</t>
+  </si>
+  <si>
+    <t>16/05/2026</t>
+  </si>
+  <si>
+    <t>IA / Herramientas</t>
+  </si>
+  <si>
+    <t>HU-033: Configuración del Entorno de IA (Ollama + LM Studio + Gemini)</t>
+  </si>
+  <si>
+    <t>Por asignar</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Medio</t>
+  </si>
+  <si>
+    <t>📋 Backlog</t>
+  </si>
+  <si>
+    <t>Preparación de entorno local</t>
+  </si>
+  <si>
+    <t>Automatización</t>
+  </si>
+  <si>
+    <t>HU-034: Flujos Base en n8n</t>
+  </si>
+  <si>
+    <t>15/06/2026</t>
+  </si>
+  <si>
+    <t>Orquestación de flujos</t>
+  </si>
+  <si>
+    <t>Backend</t>
+  </si>
+  <si>
+    <t>HU-036: Estructura Base del API (NestJS)</t>
+  </si>
+  <si>
+    <t>22/06/2026</t>
+  </si>
+  <si>
+    <t>Definición de arquitectura</t>
+  </si>
+  <si>
+    <t>Frontend</t>
+  </si>
+  <si>
+    <t>HU-037: Capa de Servicios del Frontend (Integración con API)</t>
+  </si>
+  <si>
+    <t>29/06/2026</t>
+  </si>
+  <si>
+    <t>Consumo de endpoints</t>
+  </si>
+  <si>
+    <t>IA / Training</t>
+  </si>
+  <si>
+    <t>HU-038: Fine-Tuning y Preparación de Datasets de IA</t>
+  </si>
+  <si>
+    <t>Alto</t>
+  </si>
+  <si>
+    <t>Refinamiento de datos</t>
+  </si>
+  <si>
+    <t>IA / Modelos</t>
+  </si>
+  <si>
+    <t>HU-039: Entrenamiento y Fine-Tuning de Modelos de IA</t>
+  </si>
+  <si>
+    <t>13/07/2026</t>
+  </si>
+  <si>
+    <t>Fase final de modelos</t>
+  </si>
 </sst>
 </file>
 
@@ -655,7 +793,7 @@
     <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -701,13 +839,6 @@
       <u/>
       <sz val="11"/>
       <color rgb="FF0563C1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -774,8 +905,37 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="9"/>
+      <color rgb="FF1A1A1A"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF434343"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF2C481F"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="19">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -884,8 +1044,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F8F9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="16">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -1030,21 +1202,6 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
         <color rgb="FFB8DC6E"/>
       </left>
       <right style="thin">
@@ -1118,30 +1275,118 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB8DC6E"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB8DC6E"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF80BC00"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF80BC00"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF80BC00"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF80BC00"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="42" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="41" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1154,100 +1399,182 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="8" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="16" borderId="14" xfId="16" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="16" borderId="14" xfId="16" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="13" xfId="15" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="12" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="8" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="10" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="9" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="18" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="9" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="18" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="8" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="14" xfId="17" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="11" xfId="14" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="9" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="12" xfId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="18" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="17" xfId="16" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="17" borderId="15" xfId="17" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="11" xfId="13" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="15" xfId="14" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="20" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="12" xfId="14" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="21" xfId="14" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="21" xfId="17" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="15" xfId="13" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="14" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="18" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="18" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="18" borderId="15" xfId="17" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="13" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="14" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="17" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="15" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="19"/>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="15" xfId="17" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="19" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="17" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="9" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="18" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="10" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="15" xfId="17" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="18" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="15" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" xfId="17" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="18" fillId="19" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="18" fillId="17" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="20" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="15" xfId="17" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -1539,12 +1866,12 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O33"/>
+  <dimension ref="A1:P65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" customWidth="1"/>
-    <col min="3" max="3" width="54.5703125" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="62" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.140625" customWidth="1"/>
     <col min="5" max="5" width="11.28515625" customWidth="1"/>
     <col min="6" max="6" width="67.7109375" bestFit="1" customWidth="1"/>
@@ -1559,104 +1886,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3"/>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
     </row>
     <row r="2" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="14" t="s">
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
-      <c r="O2" s="14"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
     </row>
     <row r="3" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15"/>
       <c r="B3" s="15"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="13" t="s">
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="L3" s="13"/>
-      <c r="M3" s="13"/>
-      <c r="N3" s="13"/>
-      <c r="O3" s="13"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12"/>
+      <c r="O3" s="12"/>
     </row>
     <row r="4" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="15"/>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="12"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="12"/>
-      <c r="K4" s="11" t="s">
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="11"/>
+      <c r="K4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="L4" s="11"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="11"/>
-      <c r="O4" s="11"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="9"/>
     </row>
     <row r="5" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="3"/>
-      <c r="O5" s="3"/>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
     </row>
     <row r="6" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="6" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="17" t="s">
@@ -1664,7 +1991,7 @@
       </c>
       <c r="C6" s="17"/>
       <c r="D6" s="17"/>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="6" t="s">
         <v>8</v>
       </c>
       <c r="G6" s="17" t="s">
@@ -1672,14 +1999,14 @@
       </c>
       <c r="H6" s="17"/>
       <c r="I6" s="17"/>
-      <c r="J6" s="8" t="s">
+      <c r="J6" s="6" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="17" t="s">
         <v>11</v>
       </c>
       <c r="L6" s="17"/>
-      <c r="M6" s="8" t="s">
+      <c r="M6" s="6" t="s">
         <v>12</v>
       </c>
       <c r="N6" s="17" t="s">
@@ -1688,36 +2015,36 @@
       <c r="O6" s="17"/>
     </row>
     <row r="7" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="8" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="16" t="s">
         <v>15</v>
       </c>
       <c r="C7" s="16"/>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E7" s="16" t="s">
         <v>17</v>
       </c>
       <c r="F7" s="16"/>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="8" t="s">
         <v>18</v>
       </c>
       <c r="H7" s="16" t="s">
         <v>19</v>
       </c>
       <c r="I7" s="16"/>
-      <c r="J7" s="10" t="s">
+      <c r="J7" s="8" t="s">
         <v>20</v>
       </c>
       <c r="K7" s="16">
         <f>COUNTA(A10:A32)</f>
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L7" s="16"/>
-      <c r="M7" s="10" t="s">
+      <c r="M7" s="8" t="s">
         <v>21</v>
       </c>
       <c r="N7" s="16">
@@ -1727,1129 +2054,2080 @@
       <c r="O7" s="16"/>
     </row>
     <row r="8" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="12"/>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
-      <c r="N8" s="12"/>
-      <c r="O8" s="12"/>
-    </row>
-    <row r="9" spans="1:15" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="13" t="s">
+      <c r="A8" s="10"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10"/>
+    </row>
+    <row r="9" spans="1:15" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="G9" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="H9" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="I9" s="13" t="s">
+      <c r="I9" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="J9" s="13" t="s">
+      <c r="J9" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="K9" s="13" t="s">
+      <c r="K9" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="L9" s="13" t="s">
+      <c r="L9" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="M9" s="13" t="s">
+      <c r="M9" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="N9" s="13" t="s">
+      <c r="N9" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="O9" s="13" t="s">
+      <c r="O9" s="31" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="11">
+      <c r="A10" s="22">
         <v>1</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="C10" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="25" t="s">
+      <c r="D10" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="26">
+      <c r="E10" s="34">
         <v>3</v>
       </c>
-      <c r="F10" s="24" t="s">
+      <c r="F10" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="G10" s="27" t="s">
+      <c r="G10" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="H10" s="27" t="s">
+      <c r="H10" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="I10" s="27" t="s">
+      <c r="I10" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="26" t="s">
+      <c r="J10" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="K10" s="26" t="s">
+      <c r="K10" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L10" s="26">
+      <c r="L10" s="34">
         <v>1</v>
       </c>
-      <c r="M10" s="26" t="s">
+      <c r="M10" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="N10" s="26" t="s">
+      <c r="N10" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O10" s="24" t="s">
+      <c r="O10" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="15">
+      <c r="A11" s="36">
         <v>2</v>
       </c>
-      <c r="B11" s="24" t="s">
+      <c r="B11" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="28" t="s">
+      <c r="C11" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="25" t="s">
+      <c r="D11" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="26">
+      <c r="E11" s="34">
         <v>3</v>
       </c>
-      <c r="F11" s="28" t="s">
+      <c r="F11" s="37" t="s">
         <v>49</v>
       </c>
-      <c r="G11" s="27" t="s">
+      <c r="G11" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="H11" s="27" t="s">
+      <c r="H11" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="I11" s="27" t="s">
+      <c r="I11" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="J11" s="29" t="s">
+      <c r="J11" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="K11" s="26" t="s">
+      <c r="K11" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L11" s="26">
+      <c r="L11" s="34">
         <v>1</v>
       </c>
-      <c r="M11" s="26" t="s">
+      <c r="M11" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="N11" s="26" t="s">
+      <c r="N11" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O11" s="24" t="s">
+      <c r="O11" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11">
+      <c r="A12" s="22">
         <v>3</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="24" t="s">
+      <c r="C12" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="D12" s="25" t="s">
+      <c r="D12" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="E12" s="26">
+      <c r="E12" s="34">
         <v>3</v>
       </c>
-      <c r="F12" s="24" t="s">
+      <c r="F12" s="32" t="s">
         <v>51</v>
       </c>
-      <c r="G12" s="27" t="s">
+      <c r="G12" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="H12" s="27" t="s">
+      <c r="H12" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="I12" s="27" t="s">
+      <c r="I12" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="J12" s="26" t="s">
+      <c r="J12" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="K12" s="26" t="s">
+      <c r="K12" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L12" s="26">
+      <c r="L12" s="34">
         <v>1</v>
       </c>
-      <c r="M12" s="26" t="s">
+      <c r="M12" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="N12" s="26" t="s">
+      <c r="N12" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O12" s="24" t="s">
+      <c r="O12" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="15">
+      <c r="A13" s="36">
         <v>4</v>
       </c>
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="28" t="s">
+      <c r="C13" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="D13" s="25" t="s">
+      <c r="D13" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="E13" s="26">
+      <c r="E13" s="34">
         <v>3</v>
       </c>
-      <c r="F13" s="28" t="s">
+      <c r="F13" s="37" t="s">
         <v>53</v>
       </c>
-      <c r="G13" s="27" t="s">
+      <c r="G13" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="H13" s="27" t="s">
+      <c r="H13" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="I13" s="27" t="s">
+      <c r="I13" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="26" t="s">
+      <c r="J13" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="K13" s="26" t="s">
+      <c r="K13" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L13" s="26">
+      <c r="L13" s="34">
         <v>1</v>
       </c>
-      <c r="M13" s="26" t="s">
+      <c r="M13" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="N13" s="26" t="s">
+      <c r="N13" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O13" s="24" t="s">
+      <c r="O13" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="11">
+      <c r="A14" s="22">
         <v>5</v>
       </c>
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="24" t="s">
+      <c r="C14" s="32" t="s">
         <v>54</v>
       </c>
-      <c r="D14" s="25" t="s">
+      <c r="D14" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="26">
+      <c r="E14" s="34">
         <v>3</v>
       </c>
-      <c r="F14" s="24" t="s">
+      <c r="F14" s="32" t="s">
         <v>55</v>
       </c>
-      <c r="G14" s="27" t="s">
+      <c r="G14" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="H14" s="27" t="s">
+      <c r="H14" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="I14" s="27" t="s">
+      <c r="I14" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="J14" s="29" t="s">
+      <c r="J14" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="K14" s="26" t="s">
+      <c r="K14" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L14" s="26">
+      <c r="L14" s="34">
         <v>1</v>
       </c>
-      <c r="M14" s="26" t="s">
+      <c r="M14" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="N14" s="26" t="s">
+      <c r="N14" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O14" s="24" t="s">
+      <c r="O14" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="15">
+      <c r="A15" s="36">
         <v>6</v>
       </c>
-      <c r="B15" s="24" t="s">
+      <c r="B15" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="28" t="s">
+      <c r="C15" s="37" t="s">
         <v>56</v>
       </c>
-      <c r="D15" s="25" t="s">
+      <c r="D15" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="E15" s="26">
+      <c r="E15" s="34">
         <v>3</v>
       </c>
-      <c r="F15" s="28" t="s">
+      <c r="F15" s="37" t="s">
         <v>57</v>
       </c>
-      <c r="G15" s="27" t="s">
+      <c r="G15" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="H15" s="27" t="s">
+      <c r="H15" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="I15" s="27" t="s">
+      <c r="I15" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="J15" s="26" t="s">
+      <c r="J15" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="K15" s="26" t="s">
+      <c r="K15" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L15" s="26">
+      <c r="L15" s="34">
         <v>1</v>
       </c>
-      <c r="M15" s="26" t="s">
+      <c r="M15" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="N15" s="26" t="s">
+      <c r="N15" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O15" s="24" t="s">
+      <c r="O15" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="11">
+      <c r="A16" s="22">
         <v>7</v>
       </c>
-      <c r="B16" s="24" t="s">
+      <c r="B16" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="24" t="s">
+      <c r="C16" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="D16" s="25" t="s">
+      <c r="D16" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="E16" s="26">
+      <c r="E16" s="34">
         <v>3</v>
       </c>
-      <c r="F16" s="24" t="s">
+      <c r="F16" s="32" t="s">
         <v>46</v>
       </c>
-      <c r="G16" s="27" t="s">
+      <c r="G16" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="H16" s="27" t="s">
+      <c r="H16" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="I16" s="27" t="s">
+      <c r="I16" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="J16" s="26" t="s">
+      <c r="J16" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="K16" s="26" t="s">
+      <c r="K16" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L16" s="26">
+      <c r="L16" s="34">
         <v>1</v>
       </c>
-      <c r="M16" s="26" t="s">
+      <c r="M16" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="N16" s="26" t="s">
+      <c r="N16" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O16" s="24" t="s">
+      <c r="O16" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="15">
+      <c r="A17" s="36">
         <v>10</v>
       </c>
-      <c r="B17" s="28" t="s">
+      <c r="B17" s="37" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="28" t="s">
+      <c r="C17" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="D17" s="25" t="s">
+      <c r="D17" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="E17" s="26">
+      <c r="E17" s="34">
         <v>3</v>
       </c>
-      <c r="F17" s="28" t="s">
+      <c r="F17" s="37" t="s">
         <v>62</v>
       </c>
-      <c r="G17" s="27" t="s">
+      <c r="G17" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="H17" s="27" t="s">
+      <c r="H17" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="I17" s="27" t="s">
+      <c r="I17" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="J17" s="26" t="s">
+      <c r="J17" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="K17" s="26" t="s">
+      <c r="K17" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L17" s="26">
+      <c r="L17" s="34">
         <v>1</v>
       </c>
-      <c r="M17" s="26" t="s">
+      <c r="M17" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="N17" s="26" t="s">
+      <c r="N17" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O17" s="24" t="s">
+      <c r="O17" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="18" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="11">
+      <c r="A18" s="22">
         <v>11</v>
       </c>
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="C18" s="24" t="s">
+      <c r="C18" s="32" t="s">
         <v>66</v>
       </c>
-      <c r="D18" s="25" t="s">
+      <c r="D18" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="E18" s="26">
+      <c r="E18" s="34">
         <v>3</v>
       </c>
-      <c r="F18" s="24" t="s">
+      <c r="F18" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="G18" s="27" t="s">
+      <c r="G18" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="H18" s="27" t="s">
+      <c r="H18" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="I18" s="27" t="s">
+      <c r="I18" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="J18" s="29" t="s">
+      <c r="J18" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="K18" s="26" t="s">
+      <c r="K18" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L18" s="26">
+      <c r="L18" s="34">
         <v>1</v>
       </c>
-      <c r="M18" s="26" t="s">
+      <c r="M18" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="N18" s="26" t="s">
+      <c r="N18" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O18" s="24" t="s">
+      <c r="O18" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="15">
+      <c r="A19" s="36">
         <v>12</v>
       </c>
-      <c r="B19" s="28" t="s">
+      <c r="B19" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="C19" s="28" t="s">
+      <c r="C19" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="D19" s="25" t="s">
+      <c r="D19" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="E19" s="26">
+      <c r="E19" s="34">
         <v>3</v>
       </c>
-      <c r="F19" s="28" t="s">
+      <c r="F19" s="37" t="s">
         <v>70</v>
       </c>
-      <c r="G19" s="27" t="s">
+      <c r="G19" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="H19" s="27" t="s">
+      <c r="H19" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="I19" s="27" t="s">
+      <c r="I19" s="35" t="s">
         <v>71</v>
       </c>
-      <c r="J19" s="26" t="s">
+      <c r="J19" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="K19" s="26" t="s">
+      <c r="K19" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L19" s="26">
+      <c r="L19" s="34">
         <v>1</v>
       </c>
-      <c r="M19" s="26" t="s">
+      <c r="M19" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="N19" s="26" t="s">
+      <c r="N19" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O19" s="24" t="s">
+      <c r="O19" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="20" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="11">
+      <c r="A20" s="22">
         <v>13</v>
       </c>
-      <c r="B20" s="24" t="s">
+      <c r="B20" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="C20" s="24" t="s">
+      <c r="C20" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="D20" s="25" t="s">
+      <c r="D20" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="E20" s="26">
+      <c r="E20" s="34">
         <v>3</v>
       </c>
-      <c r="F20" s="24" t="s">
+      <c r="F20" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="G20" s="27" t="s">
+      <c r="G20" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="H20" s="27" t="s">
+      <c r="H20" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="I20" s="27" t="s">
+      <c r="I20" s="35" t="s">
         <v>75</v>
       </c>
-      <c r="J20" s="26" t="s">
+      <c r="J20" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="K20" s="26" t="s">
+      <c r="K20" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L20" s="26">
+      <c r="L20" s="34">
         <v>1</v>
       </c>
-      <c r="M20" s="26" t="s">
+      <c r="M20" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="N20" s="26" t="s">
+      <c r="N20" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O20" s="24" t="s">
+      <c r="O20" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="15">
+      <c r="A21" s="36">
         <v>14</v>
       </c>
-      <c r="B21" s="28" t="s">
+      <c r="B21" s="37" t="s">
         <v>76</v>
       </c>
-      <c r="C21" s="28" t="s">
+      <c r="C21" s="37" t="s">
         <v>77</v>
       </c>
-      <c r="D21" s="25" t="s">
+      <c r="D21" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="E21" s="26">
+      <c r="E21" s="34">
         <v>3</v>
       </c>
-      <c r="F21" s="28" t="s">
+      <c r="F21" s="37" t="s">
         <v>70</v>
       </c>
-      <c r="G21" s="27" t="s">
+      <c r="G21" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="H21" s="27" t="s">
+      <c r="H21" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="I21" s="27" t="s">
+      <c r="I21" s="35" t="s">
         <v>78</v>
       </c>
-      <c r="J21" s="29" t="s">
+      <c r="J21" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="K21" s="26" t="s">
+      <c r="K21" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L21" s="26">
+      <c r="L21" s="34">
         <v>1</v>
       </c>
-      <c r="M21" s="29" t="s">
+      <c r="M21" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="N21" s="26" t="s">
+      <c r="N21" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O21" s="24" t="s">
+      <c r="O21" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="11">
+      <c r="A22" s="22">
         <v>15</v>
       </c>
-      <c r="B22" s="24" t="s">
+      <c r="B22" s="32" t="s">
         <v>76</v>
       </c>
-      <c r="C22" s="24" t="s">
+      <c r="C22" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="D22" s="25" t="s">
+      <c r="D22" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="E22" s="26">
+      <c r="E22" s="34">
         <v>3</v>
       </c>
-      <c r="F22" s="24" t="s">
+      <c r="F22" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="G22" s="27" t="s">
+      <c r="G22" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="H22" s="27" t="s">
+      <c r="H22" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="I22" s="27" t="s">
+      <c r="I22" s="35" t="s">
         <v>80</v>
       </c>
-      <c r="J22" s="26" t="s">
+      <c r="J22" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="K22" s="26" t="s">
+      <c r="K22" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L22" s="26">
+      <c r="L22" s="34">
         <v>1</v>
       </c>
-      <c r="M22" s="26" t="s">
+      <c r="M22" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="N22" s="26" t="s">
+      <c r="N22" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O22" s="24" t="s">
+      <c r="O22" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="15">
+      <c r="A23" s="36">
         <v>16</v>
       </c>
-      <c r="B23" s="28" t="s">
+      <c r="B23" s="37" t="s">
         <v>76</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="37" t="s">
         <v>81</v>
       </c>
-      <c r="D23" s="25" t="s">
+      <c r="D23" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="E23" s="26">
+      <c r="E23" s="34">
         <v>3</v>
       </c>
-      <c r="F23" s="28" t="s">
+      <c r="F23" s="37" t="s">
         <v>62</v>
       </c>
-      <c r="G23" s="27" t="s">
+      <c r="G23" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="H23" s="27" t="s">
+      <c r="H23" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="I23" s="27" t="s">
+      <c r="I23" s="35" t="s">
         <v>82</v>
       </c>
-      <c r="J23" s="26" t="s">
+      <c r="J23" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="K23" s="26" t="s">
+      <c r="K23" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L23" s="26">
+      <c r="L23" s="34">
         <v>1</v>
       </c>
-      <c r="M23" s="29" t="s">
+      <c r="M23" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="N23" s="26" t="s">
+      <c r="N23" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O23" s="24" t="s">
+      <c r="O23" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="11">
+      <c r="A24" s="22">
         <v>17</v>
       </c>
-      <c r="B24" s="24" t="s">
+      <c r="B24" s="32" t="s">
         <v>76</v>
       </c>
-      <c r="C24" s="24" t="s">
+      <c r="C24" s="32" t="s">
         <v>83</v>
       </c>
-      <c r="D24" s="25" t="s">
+      <c r="D24" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="E24" s="26">
+      <c r="E24" s="34">
         <v>3</v>
       </c>
-      <c r="F24" s="24" t="s">
+      <c r="F24" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="G24" s="27" t="s">
+      <c r="G24" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="H24" s="27" t="s">
+      <c r="H24" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="I24" s="27" t="s">
+      <c r="I24" s="35" t="s">
         <v>84</v>
       </c>
-      <c r="J24" s="29" t="s">
+      <c r="J24" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="K24" s="26" t="s">
+      <c r="K24" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L24" s="26">
+      <c r="L24" s="34">
         <v>1</v>
       </c>
-      <c r="M24" s="26" t="s">
+      <c r="M24" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="N24" s="26" t="s">
+      <c r="N24" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O24" s="24" t="s">
+      <c r="O24" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="15">
+      <c r="A25" s="36">
         <v>18</v>
       </c>
-      <c r="B25" s="28" t="s">
+      <c r="B25" s="37" t="s">
         <v>76</v>
       </c>
-      <c r="C25" s="28" t="s">
+      <c r="C25" s="37" t="s">
         <v>85</v>
       </c>
-      <c r="D25" s="25" t="s">
+      <c r="D25" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="E25" s="26">
+      <c r="E25" s="34">
         <v>3</v>
       </c>
-      <c r="F25" s="28" t="s">
+      <c r="F25" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="G25" s="27" t="s">
+      <c r="G25" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="H25" s="27" t="s">
+      <c r="H25" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="I25" s="27" t="s">
+      <c r="I25" s="35" t="s">
         <v>87</v>
       </c>
-      <c r="J25" s="26" t="s">
+      <c r="J25" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="K25" s="26" t="s">
+      <c r="K25" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L25" s="26">
+      <c r="L25" s="34">
         <v>1</v>
       </c>
-      <c r="M25" s="29" t="s">
+      <c r="M25" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="N25" s="26" t="s">
+      <c r="N25" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O25" s="24" t="s">
+      <c r="O25" s="32" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="26" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="11">
+      <c r="A26" s="22">
         <v>19</v>
       </c>
-      <c r="B26" s="24" t="s">
+      <c r="B26" s="32" t="s">
         <v>76</v>
       </c>
-      <c r="C26" s="24" t="s">
+      <c r="C26" s="32" t="s">
         <v>89</v>
       </c>
-      <c r="D26" s="25" t="s">
+      <c r="D26" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="E26" s="26">
+      <c r="E26" s="34">
         <v>3</v>
       </c>
-      <c r="F26" s="24" t="s">
+      <c r="F26" s="32" t="s">
         <v>90</v>
       </c>
-      <c r="G26" s="27" t="s">
+      <c r="G26" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="H26" s="27" t="s">
+      <c r="H26" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="I26" s="27" t="s">
+      <c r="I26" s="35" t="s">
         <v>91</v>
       </c>
-      <c r="J26" s="26" t="s">
+      <c r="J26" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="K26" s="26" t="s">
+      <c r="K26" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L26" s="26">
+      <c r="L26" s="34">
         <v>1</v>
       </c>
-      <c r="M26" s="26" t="s">
+      <c r="M26" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="N26" s="26" t="s">
+      <c r="N26" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O26" s="24" t="s">
+      <c r="O26" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="27" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="15">
+      <c r="A27" s="36">
         <v>20</v>
       </c>
-      <c r="B27" s="28" t="s">
+      <c r="B27" s="37" t="s">
         <v>76</v>
       </c>
-      <c r="C27" s="28" t="s">
+      <c r="C27" s="37" t="s">
         <v>92</v>
       </c>
-      <c r="D27" s="25" t="s">
+      <c r="D27" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="E27" s="26">
+      <c r="E27" s="34">
         <v>3</v>
       </c>
-      <c r="F27" s="28" t="s">
+      <c r="F27" s="37" t="s">
         <v>93</v>
       </c>
-      <c r="G27" s="27" t="s">
+      <c r="G27" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="H27" s="27" t="s">
+      <c r="H27" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="I27" s="27" t="s">
+      <c r="I27" s="35" t="s">
         <v>94</v>
       </c>
-      <c r="J27" s="29" t="s">
+      <c r="J27" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="K27" s="26" t="s">
+      <c r="K27" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L27" s="29">
+      <c r="L27" s="38">
         <v>1</v>
       </c>
-      <c r="M27" s="29" t="s">
+      <c r="M27" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="N27" s="26" t="s">
+      <c r="N27" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O27" s="24" t="s">
+      <c r="O27" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="28" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="11"/>
-      <c r="B28" s="24" t="s">
+      <c r="A28" s="36">
+        <v>21</v>
+      </c>
+      <c r="B28" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="C28" s="24" t="s">
+      <c r="C28" s="32" t="s">
         <v>142</v>
       </c>
-      <c r="D28" s="30" t="s">
+      <c r="D28" s="39" t="s">
         <v>154</v>
       </c>
-      <c r="E28" s="26">
+      <c r="E28" s="34">
         <v>3</v>
       </c>
-      <c r="F28" s="24" t="s">
+      <c r="F28" s="32" t="s">
         <v>147</v>
       </c>
-      <c r="G28" s="27">
+      <c r="G28" s="35">
         <v>46086</v>
       </c>
-      <c r="H28" s="27">
+      <c r="H28" s="35">
         <v>46270</v>
       </c>
-      <c r="I28" s="27">
+      <c r="I28" s="35">
         <v>46271</v>
       </c>
-      <c r="J28" s="26" t="s">
+      <c r="J28" s="34" t="s">
         <v>145</v>
       </c>
-      <c r="K28" s="26" t="s">
+      <c r="K28" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L28" s="26">
+      <c r="L28" s="34">
         <v>1</v>
       </c>
-      <c r="M28" s="29" t="s">
+      <c r="M28" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="N28" s="26" t="s">
+      <c r="N28" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O28" s="24" t="s">
+      <c r="O28" s="32" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="29" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="15"/>
-      <c r="B29" s="28" t="s">
+      <c r="A29" s="22">
+        <v>22</v>
+      </c>
+      <c r="B29" s="37" t="s">
         <v>152</v>
       </c>
-      <c r="C29" s="28" t="s">
+      <c r="C29" s="37" t="s">
         <v>143</v>
       </c>
-      <c r="D29" s="30" t="s">
+      <c r="D29" s="39" t="s">
         <v>154</v>
       </c>
-      <c r="E29" s="26">
+      <c r="E29" s="34">
         <v>3</v>
       </c>
-      <c r="F29" s="24" t="s">
+      <c r="F29" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="G29" s="27">
+      <c r="G29" s="35">
         <v>46086</v>
       </c>
-      <c r="H29" s="27">
+      <c r="H29" s="35">
         <v>46270</v>
       </c>
-      <c r="I29" s="27">
+      <c r="I29" s="35">
         <v>46271</v>
       </c>
-      <c r="J29" s="26" t="s">
+      <c r="J29" s="34" t="s">
         <v>145</v>
       </c>
-      <c r="K29" s="26" t="s">
+      <c r="K29" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="L29" s="26">
+      <c r="L29" s="34">
         <v>1</v>
       </c>
-      <c r="M29" s="29" t="s">
+      <c r="M29" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="N29" s="26" t="s">
+      <c r="N29" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O29" s="24" t="s">
+      <c r="O29" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="30" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="11"/>
-      <c r="B30" s="28" t="s">
+      <c r="A30" s="36">
+        <v>23</v>
+      </c>
+      <c r="B30" s="37" t="s">
         <v>152</v>
       </c>
-      <c r="C30" s="24" t="s">
+      <c r="C30" s="32" t="s">
         <v>144</v>
       </c>
-      <c r="D30" s="30" t="s">
+      <c r="D30" s="39" t="s">
         <v>154</v>
       </c>
-      <c r="E30" s="26">
+      <c r="E30" s="34">
         <v>3</v>
       </c>
-      <c r="F30" s="24" t="s">
+      <c r="F30" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="G30" s="27">
+      <c r="G30" s="35">
         <v>46086</v>
       </c>
-      <c r="H30" s="27">
+      <c r="H30" s="35">
         <v>46270</v>
       </c>
-      <c r="I30" s="27">
+      <c r="I30" s="35">
         <v>46271</v>
       </c>
-      <c r="J30" s="26" t="s">
+      <c r="J30" s="34" t="s">
         <v>145</v>
       </c>
-      <c r="K30" s="26" t="s">
+      <c r="K30" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="L30" s="29">
+      <c r="L30" s="38">
         <v>1</v>
       </c>
-      <c r="M30" s="29" t="s">
+      <c r="M30" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="N30" s="26" t="s">
+      <c r="N30" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O30" s="24" t="s">
+      <c r="O30" s="32" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="31" spans="1:15" s="23" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="19"/>
-      <c r="B31" s="20" t="s">
+    <row r="31" spans="1:15" s="15" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="61">
+        <v>24</v>
+      </c>
+      <c r="B31" s="41" t="s">
         <v>153</v>
       </c>
-      <c r="C31" s="20" t="s">
+      <c r="C31" s="41" t="s">
         <v>148</v>
       </c>
-      <c r="D31" s="20"/>
-      <c r="E31" s="21">
+      <c r="D31" s="41"/>
+      <c r="E31" s="42">
         <v>3</v>
       </c>
-      <c r="F31" s="20" t="s">
+      <c r="F31" s="41" t="s">
         <v>149</v>
       </c>
-      <c r="G31" s="22">
+      <c r="G31" s="43">
         <v>46086</v>
       </c>
-      <c r="H31" s="22">
+      <c r="H31" s="43">
         <v>46270</v>
       </c>
-      <c r="I31" s="22"/>
-      <c r="J31" s="21" t="s">
+      <c r="I31" s="43"/>
+      <c r="J31" s="42" t="s">
         <v>145</v>
       </c>
-      <c r="K31" s="21" t="s">
+      <c r="K31" s="42" t="s">
         <v>44</v>
       </c>
-      <c r="L31" s="21">
+      <c r="L31" s="42">
         <v>1</v>
       </c>
-      <c r="M31" s="19" t="s">
+      <c r="M31" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="N31" s="21" t="s">
+      <c r="N31" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="O31" s="20" t="s">
+      <c r="O31" s="41" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="32" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="11"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="11"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="11"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="11"/>
-      <c r="J32" s="11"/>
-      <c r="K32" s="11"/>
-      <c r="L32" s="11"/>
-      <c r="M32" s="11"/>
-      <c r="N32" s="11"/>
-      <c r="O32" s="14"/>
-    </row>
-    <row r="33" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="18" t="s">
+    <row r="32" spans="1:15" s="25" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="45">
+        <v>25</v>
+      </c>
+      <c r="B32" s="46" t="s">
+        <v>153</v>
+      </c>
+      <c r="C32" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="D32" s="47" t="s">
+        <v>162</v>
+      </c>
+      <c r="E32" s="45">
+        <v>3</v>
+      </c>
+      <c r="F32" s="46" t="s">
+        <v>57</v>
+      </c>
+      <c r="G32" s="48">
+        <v>46270</v>
+      </c>
+      <c r="H32" s="48" t="s">
+        <v>155</v>
+      </c>
+      <c r="I32" s="48"/>
+      <c r="J32" s="45" t="s">
+        <v>145</v>
+      </c>
+      <c r="K32" s="45" t="s">
+        <v>44</v>
+      </c>
+      <c r="L32" s="45">
+        <v>1</v>
+      </c>
+      <c r="M32" s="49"/>
+      <c r="N32" s="45"/>
+      <c r="O32" s="46"/>
+    </row>
+    <row r="33" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="22">
+        <v>26</v>
+      </c>
+      <c r="B33" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="C33" s="50" t="s">
+        <v>157</v>
+      </c>
+      <c r="D33" s="51" t="s">
+        <v>162</v>
+      </c>
+      <c r="E33" s="52">
+        <v>3</v>
+      </c>
+      <c r="F33" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="G33" s="52" t="s">
+        <v>158</v>
+      </c>
+      <c r="H33" s="52" t="s">
+        <v>159</v>
+      </c>
+      <c r="I33" s="48"/>
+      <c r="J33" s="45"/>
+      <c r="K33" s="45"/>
+      <c r="L33" s="45"/>
+      <c r="M33" s="22"/>
+      <c r="N33" s="22"/>
+      <c r="O33" s="23"/>
+      <c r="P33" s="26"/>
+    </row>
+    <row r="34" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="36">
+        <v>27</v>
+      </c>
+      <c r="B34" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="C34" s="53" t="s">
+        <v>160</v>
+      </c>
+      <c r="D34" s="47" t="s">
+        <v>162</v>
+      </c>
+      <c r="E34" s="54">
+        <v>3</v>
+      </c>
+      <c r="F34" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="G34" s="54" t="s">
+        <v>158</v>
+      </c>
+      <c r="H34" s="54" t="s">
+        <v>159</v>
+      </c>
+      <c r="I34" s="22"/>
+      <c r="J34" s="22"/>
+      <c r="K34" s="22"/>
+      <c r="L34" s="22"/>
+      <c r="M34" s="22"/>
+      <c r="N34" s="22"/>
+      <c r="O34" s="23"/>
+      <c r="P34" s="26"/>
+    </row>
+    <row r="35" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="22">
+        <v>28</v>
+      </c>
+      <c r="B35" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="C35" s="50" t="s">
+        <v>161</v>
+      </c>
+      <c r="D35" s="47" t="s">
+        <v>162</v>
+      </c>
+      <c r="E35" s="52">
+        <v>3</v>
+      </c>
+      <c r="F35" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="G35" s="52" t="s">
+        <v>163</v>
+      </c>
+      <c r="H35" s="52" t="s">
+        <v>164</v>
+      </c>
+      <c r="I35" s="22"/>
+      <c r="J35" s="22"/>
+      <c r="K35" s="22"/>
+      <c r="L35" s="22"/>
+      <c r="M35" s="22"/>
+      <c r="N35" s="22"/>
+      <c r="O35" s="23"/>
+      <c r="P35" s="26"/>
+    </row>
+    <row r="36" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="36">
+        <v>29</v>
+      </c>
+      <c r="B36" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="C36" s="53" t="s">
+        <v>165</v>
+      </c>
+      <c r="D36" s="51" t="s">
+        <v>162</v>
+      </c>
+      <c r="E36" s="54">
+        <v>3</v>
+      </c>
+      <c r="F36" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="G36" s="54" t="s">
+        <v>163</v>
+      </c>
+      <c r="H36" s="54" t="s">
+        <v>164</v>
+      </c>
+      <c r="I36" s="22"/>
+      <c r="J36" s="22"/>
+      <c r="K36" s="22"/>
+      <c r="L36" s="22"/>
+      <c r="M36" s="22"/>
+      <c r="N36" s="22"/>
+      <c r="O36" s="23"/>
+      <c r="P36" s="26"/>
+    </row>
+    <row r="37" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="36">
+        <v>30</v>
+      </c>
+      <c r="B37" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="C37" s="50" t="s">
+        <v>166</v>
+      </c>
+      <c r="D37" s="47" t="s">
+        <v>162</v>
+      </c>
+      <c r="E37" s="52">
+        <v>3</v>
+      </c>
+      <c r="F37" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="G37" s="52" t="s">
+        <v>164</v>
+      </c>
+      <c r="H37" s="55">
+        <v>46028</v>
+      </c>
+      <c r="I37" s="22"/>
+      <c r="J37" s="22"/>
+      <c r="K37" s="22"/>
+      <c r="L37" s="22"/>
+      <c r="M37" s="22"/>
+      <c r="N37" s="22"/>
+      <c r="O37" s="23"/>
+      <c r="P37" s="26"/>
+    </row>
+    <row r="38" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="22">
+        <v>31</v>
+      </c>
+      <c r="B38" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="C38" s="53" t="s">
+        <v>167</v>
+      </c>
+      <c r="D38" s="51" t="s">
+        <v>162</v>
+      </c>
+      <c r="E38" s="54">
+        <v>3</v>
+      </c>
+      <c r="F38" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="G38" s="54" t="s">
+        <v>164</v>
+      </c>
+      <c r="H38" s="56">
+        <v>46028</v>
+      </c>
+      <c r="I38" s="22"/>
+      <c r="J38" s="22"/>
+      <c r="K38" s="22"/>
+      <c r="L38" s="22"/>
+      <c r="M38" s="22"/>
+      <c r="N38" s="22"/>
+      <c r="O38" s="23"/>
+      <c r="P38" s="26"/>
+    </row>
+    <row r="39" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="36">
+        <v>32</v>
+      </c>
+      <c r="B39" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="C39" s="50" t="s">
+        <v>168</v>
+      </c>
+      <c r="D39" s="47" t="s">
+        <v>162</v>
+      </c>
+      <c r="E39" s="52">
+        <v>3</v>
+      </c>
+      <c r="F39" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="G39" s="55">
+        <v>46028</v>
+      </c>
+      <c r="H39" s="55">
+        <v>46240</v>
+      </c>
+      <c r="I39" s="22"/>
+      <c r="J39" s="22"/>
+      <c r="K39" s="22"/>
+      <c r="L39" s="22"/>
+      <c r="M39" s="22"/>
+      <c r="N39" s="22"/>
+      <c r="O39" s="23"/>
+      <c r="P39" s="26"/>
+    </row>
+    <row r="40" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="22">
+        <v>33</v>
+      </c>
+      <c r="B40" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="C40" s="53" t="s">
+        <v>169</v>
+      </c>
+      <c r="D40" s="51" t="s">
+        <v>162</v>
+      </c>
+      <c r="E40" s="54">
+        <v>3</v>
+      </c>
+      <c r="F40" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="G40" s="56">
+        <v>46028</v>
+      </c>
+      <c r="H40" s="56">
+        <v>46240</v>
+      </c>
+      <c r="I40" s="22"/>
+      <c r="J40" s="22"/>
+      <c r="K40" s="22"/>
+      <c r="L40" s="22"/>
+      <c r="M40" s="22"/>
+      <c r="N40" s="22"/>
+      <c r="O40" s="23"/>
+      <c r="P40" s="26"/>
+    </row>
+    <row r="41" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="36">
+        <v>34</v>
+      </c>
+      <c r="B41" s="50" t="s">
+        <v>170</v>
+      </c>
+      <c r="C41" s="50" t="s">
+        <v>171</v>
+      </c>
+      <c r="D41" s="47" t="s">
+        <v>162</v>
+      </c>
+      <c r="E41" s="52">
+        <v>3</v>
+      </c>
+      <c r="F41" s="50" t="s">
+        <v>172</v>
+      </c>
+      <c r="G41" s="55">
+        <v>46270</v>
+      </c>
+      <c r="H41" s="52" t="s">
+        <v>173</v>
+      </c>
+      <c r="I41" s="22"/>
+      <c r="J41" s="22"/>
+      <c r="K41" s="22"/>
+      <c r="L41" s="22"/>
+      <c r="M41" s="22"/>
+      <c r="N41" s="22"/>
+      <c r="O41" s="23"/>
+      <c r="P41" s="26"/>
+    </row>
+    <row r="42" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="22">
+        <v>35</v>
+      </c>
+      <c r="B42" s="57" t="s">
+        <v>174</v>
+      </c>
+      <c r="C42" s="57" t="s">
+        <v>175</v>
+      </c>
+      <c r="D42" s="51" t="s">
+        <v>162</v>
+      </c>
+      <c r="E42" s="58">
+        <v>3</v>
+      </c>
+      <c r="F42" s="57" t="s">
+        <v>176</v>
+      </c>
+      <c r="G42" s="59">
+        <v>46240</v>
+      </c>
+      <c r="H42" s="59">
+        <v>46362</v>
+      </c>
+      <c r="I42" s="57" t="s">
+        <v>177</v>
+      </c>
+      <c r="J42" s="57" t="s">
+        <v>178</v>
+      </c>
+      <c r="K42" s="57" t="s">
+        <v>44</v>
+      </c>
+      <c r="L42" s="58">
+        <v>0</v>
+      </c>
+      <c r="M42" s="57" t="s">
+        <v>179</v>
+      </c>
+      <c r="N42" s="57" t="s">
+        <v>177</v>
+      </c>
+      <c r="O42" s="60" t="s">
+        <v>180</v>
+      </c>
+      <c r="P42" s="27"/>
+    </row>
+    <row r="43" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="36">
+        <v>36</v>
+      </c>
+      <c r="B43" s="57" t="s">
+        <v>181</v>
+      </c>
+      <c r="C43" s="57" t="s">
+        <v>182</v>
+      </c>
+      <c r="D43" s="47" t="s">
+        <v>162</v>
+      </c>
+      <c r="E43" s="58">
+        <v>3</v>
+      </c>
+      <c r="F43" s="57" t="s">
+        <v>176</v>
+      </c>
+      <c r="G43" s="59">
+        <v>46240</v>
+      </c>
+      <c r="H43" s="58" t="s">
+        <v>183</v>
+      </c>
+      <c r="I43" s="57" t="s">
+        <v>177</v>
+      </c>
+      <c r="J43" s="57" t="s">
+        <v>43</v>
+      </c>
+      <c r="K43" s="57" t="s">
+        <v>44</v>
+      </c>
+      <c r="L43" s="58">
+        <v>0</v>
+      </c>
+      <c r="M43" s="57" t="s">
+        <v>179</v>
+      </c>
+      <c r="N43" s="57" t="s">
+        <v>177</v>
+      </c>
+      <c r="O43" s="60" t="s">
+        <v>184</v>
+      </c>
+      <c r="P43" s="27"/>
+    </row>
+    <row r="44" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="22">
+        <v>37</v>
+      </c>
+      <c r="B44" s="57" t="s">
+        <v>185</v>
+      </c>
+      <c r="C44" s="57" t="s">
+        <v>186</v>
+      </c>
+      <c r="D44" s="51" t="s">
+        <v>162</v>
+      </c>
+      <c r="E44" s="58">
+        <v>3</v>
+      </c>
+      <c r="F44" s="57" t="s">
+        <v>176</v>
+      </c>
+      <c r="G44" s="58" t="s">
+        <v>183</v>
+      </c>
+      <c r="H44" s="58" t="s">
+        <v>187</v>
+      </c>
+      <c r="I44" s="57" t="s">
+        <v>177</v>
+      </c>
+      <c r="J44" s="57" t="s">
+        <v>43</v>
+      </c>
+      <c r="K44" s="57" t="s">
+        <v>44</v>
+      </c>
+      <c r="L44" s="58">
+        <v>0</v>
+      </c>
+      <c r="M44" s="57" t="s">
+        <v>179</v>
+      </c>
+      <c r="N44" s="57" t="s">
+        <v>177</v>
+      </c>
+      <c r="O44" s="60" t="s">
+        <v>188</v>
+      </c>
+      <c r="P44" s="27"/>
+    </row>
+    <row r="45" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="36">
+        <v>38</v>
+      </c>
+      <c r="B45" s="57" t="s">
+        <v>189</v>
+      </c>
+      <c r="C45" s="57" t="s">
+        <v>190</v>
+      </c>
+      <c r="D45" s="47" t="s">
+        <v>162</v>
+      </c>
+      <c r="E45" s="58">
+        <v>3</v>
+      </c>
+      <c r="F45" s="57" t="s">
+        <v>176</v>
+      </c>
+      <c r="G45" s="58" t="s">
+        <v>187</v>
+      </c>
+      <c r="H45" s="58" t="s">
+        <v>191</v>
+      </c>
+      <c r="I45" s="57" t="s">
+        <v>177</v>
+      </c>
+      <c r="J45" s="57" t="s">
+        <v>43</v>
+      </c>
+      <c r="K45" s="57" t="s">
+        <v>44</v>
+      </c>
+      <c r="L45" s="58">
+        <v>0</v>
+      </c>
+      <c r="M45" s="57" t="s">
+        <v>179</v>
+      </c>
+      <c r="N45" s="57" t="s">
+        <v>177</v>
+      </c>
+      <c r="O45" s="60" t="s">
+        <v>192</v>
+      </c>
+      <c r="P45" s="27"/>
+    </row>
+    <row r="46" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="36">
+        <v>39</v>
+      </c>
+      <c r="B46" s="57" t="s">
+        <v>193</v>
+      </c>
+      <c r="C46" s="57" t="s">
+        <v>194</v>
+      </c>
+      <c r="D46" s="51" t="s">
+        <v>162</v>
+      </c>
+      <c r="E46" s="58">
+        <v>3</v>
+      </c>
+      <c r="F46" s="57" t="s">
+        <v>176</v>
+      </c>
+      <c r="G46" s="58" t="s">
+        <v>191</v>
+      </c>
+      <c r="H46" s="59">
+        <v>46180</v>
+      </c>
+      <c r="I46" s="57" t="s">
+        <v>177</v>
+      </c>
+      <c r="J46" s="57" t="s">
+        <v>195</v>
+      </c>
+      <c r="K46" s="57" t="s">
+        <v>44</v>
+      </c>
+      <c r="L46" s="58">
+        <v>0</v>
+      </c>
+      <c r="M46" s="57" t="s">
+        <v>179</v>
+      </c>
+      <c r="N46" s="57" t="s">
+        <v>177</v>
+      </c>
+      <c r="O46" s="60" t="s">
+        <v>196</v>
+      </c>
+      <c r="P46" s="27"/>
+    </row>
+    <row r="47" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="22">
+        <v>40</v>
+      </c>
+      <c r="B47" s="57" t="s">
+        <v>197</v>
+      </c>
+      <c r="C47" s="57" t="s">
+        <v>198</v>
+      </c>
+      <c r="D47" s="47" t="s">
+        <v>162</v>
+      </c>
+      <c r="E47" s="58">
+        <v>3</v>
+      </c>
+      <c r="F47" s="57" t="s">
+        <v>176</v>
+      </c>
+      <c r="G47" s="59">
+        <v>46180</v>
+      </c>
+      <c r="H47" s="58" t="s">
+        <v>199</v>
+      </c>
+      <c r="I47" s="57" t="s">
+        <v>177</v>
+      </c>
+      <c r="J47" s="57" t="s">
+        <v>195</v>
+      </c>
+      <c r="K47" s="57" t="s">
+        <v>44</v>
+      </c>
+      <c r="L47" s="58">
+        <v>0</v>
+      </c>
+      <c r="M47" s="57" t="s">
+        <v>179</v>
+      </c>
+      <c r="N47" s="57" t="s">
+        <v>177</v>
+      </c>
+      <c r="O47" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P47" s="27"/>
+    </row>
+    <row r="48" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="36">
+        <v>41</v>
+      </c>
+      <c r="B48" s="23"/>
+      <c r="C48" s="23"/>
+      <c r="D48" s="51" t="s">
+        <v>162</v>
+      </c>
+      <c r="E48" s="22"/>
+      <c r="F48" s="23"/>
+      <c r="G48" s="22"/>
+      <c r="H48" s="22"/>
+      <c r="I48" s="22"/>
+      <c r="J48" s="22"/>
+      <c r="K48" s="22"/>
+      <c r="L48" s="22"/>
+      <c r="M48" s="22"/>
+      <c r="N48" s="22"/>
+      <c r="O48" s="23"/>
+      <c r="P48" s="26"/>
+    </row>
+    <row r="49" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="22">
+        <v>42</v>
+      </c>
+      <c r="B49" s="23"/>
+      <c r="C49" s="23"/>
+      <c r="D49" s="23"/>
+      <c r="E49" s="22"/>
+      <c r="F49" s="23"/>
+      <c r="G49" s="22"/>
+      <c r="H49" s="22"/>
+      <c r="I49" s="22"/>
+      <c r="J49" s="22"/>
+      <c r="K49" s="22"/>
+      <c r="L49" s="22"/>
+      <c r="M49" s="22"/>
+      <c r="N49" s="22"/>
+      <c r="O49" s="23"/>
+      <c r="P49" s="26"/>
+    </row>
+    <row r="50" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="28">
+        <v>43</v>
+      </c>
+      <c r="B50" s="29"/>
+      <c r="C50" s="29"/>
+      <c r="D50" s="29"/>
+      <c r="E50" s="30"/>
+      <c r="F50" s="29"/>
+      <c r="G50" s="30"/>
+      <c r="H50" s="30"/>
+      <c r="I50" s="30"/>
+      <c r="J50" s="30"/>
+      <c r="K50" s="30"/>
+      <c r="L50" s="30"/>
+      <c r="M50" s="30"/>
+      <c r="N50" s="30"/>
+      <c r="O50" s="29"/>
+    </row>
+    <row r="51" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="9">
+        <v>44</v>
+      </c>
+      <c r="B51" s="23"/>
+      <c r="C51" s="23"/>
+      <c r="D51" s="23"/>
+      <c r="E51" s="22"/>
+      <c r="F51" s="23"/>
+      <c r="G51" s="22"/>
+      <c r="H51" s="22"/>
+      <c r="I51" s="22"/>
+      <c r="J51" s="22"/>
+      <c r="K51" s="22"/>
+      <c r="L51" s="22"/>
+      <c r="M51" s="22"/>
+      <c r="N51" s="22"/>
+      <c r="O51" s="23"/>
+    </row>
+    <row r="52" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="12">
+        <v>45</v>
+      </c>
+      <c r="B52" s="23"/>
+      <c r="C52" s="23"/>
+      <c r="D52" s="23"/>
+      <c r="E52" s="22"/>
+      <c r="F52" s="23"/>
+      <c r="G52" s="22"/>
+      <c r="H52" s="22"/>
+      <c r="I52" s="22"/>
+      <c r="J52" s="22"/>
+      <c r="K52" s="22"/>
+      <c r="L52" s="22"/>
+      <c r="M52" s="22"/>
+      <c r="N52" s="22"/>
+      <c r="O52" s="23"/>
+    </row>
+    <row r="53" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="9">
+        <v>46</v>
+      </c>
+      <c r="B53" s="23"/>
+      <c r="C53" s="23"/>
+      <c r="D53" s="23"/>
+      <c r="E53" s="22"/>
+      <c r="F53" s="23"/>
+      <c r="G53" s="22"/>
+      <c r="H53" s="22"/>
+      <c r="I53" s="22"/>
+      <c r="J53" s="22"/>
+      <c r="K53" s="22"/>
+      <c r="L53" s="22"/>
+      <c r="M53" s="22"/>
+      <c r="N53" s="22"/>
+      <c r="O53" s="23"/>
+    </row>
+    <row r="54" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="12">
+        <v>47</v>
+      </c>
+      <c r="B54" s="23"/>
+      <c r="C54" s="23"/>
+      <c r="D54" s="23"/>
+      <c r="E54" s="22"/>
+      <c r="F54" s="23"/>
+      <c r="G54" s="22"/>
+      <c r="H54" s="22"/>
+      <c r="I54" s="22"/>
+      <c r="J54" s="22"/>
+      <c r="K54" s="22"/>
+      <c r="L54" s="22"/>
+      <c r="M54" s="22"/>
+      <c r="N54" s="22"/>
+      <c r="O54" s="23"/>
+    </row>
+    <row r="55" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="9">
+        <v>48</v>
+      </c>
+      <c r="B55" s="23"/>
+      <c r="C55" s="23"/>
+      <c r="D55" s="23"/>
+      <c r="E55" s="22"/>
+      <c r="F55" s="23"/>
+      <c r="G55" s="22"/>
+      <c r="H55" s="22"/>
+      <c r="I55" s="22"/>
+      <c r="J55" s="22"/>
+      <c r="K55" s="22"/>
+      <c r="L55" s="22"/>
+      <c r="M55" s="22"/>
+      <c r="N55" s="22"/>
+      <c r="O55" s="23"/>
+    </row>
+    <row r="56" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="12">
+        <v>49</v>
+      </c>
+      <c r="B56" s="23"/>
+      <c r="C56" s="23"/>
+      <c r="D56" s="23"/>
+      <c r="E56" s="22"/>
+      <c r="F56" s="23"/>
+      <c r="G56" s="22"/>
+      <c r="H56" s="22"/>
+      <c r="I56" s="22"/>
+      <c r="J56" s="22"/>
+      <c r="K56" s="22"/>
+      <c r="L56" s="22"/>
+      <c r="M56" s="22"/>
+      <c r="N56" s="22"/>
+      <c r="O56" s="23"/>
+    </row>
+    <row r="57" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="12">
+        <v>50</v>
+      </c>
+      <c r="B57" s="23"/>
+      <c r="C57" s="23"/>
+      <c r="D57" s="23"/>
+      <c r="E57" s="22"/>
+      <c r="F57" s="23"/>
+      <c r="G57" s="22"/>
+      <c r="H57" s="22"/>
+      <c r="I57" s="22"/>
+      <c r="J57" s="22"/>
+      <c r="K57" s="22"/>
+      <c r="L57" s="22"/>
+      <c r="M57" s="22"/>
+      <c r="N57" s="22"/>
+      <c r="O57" s="23"/>
+    </row>
+    <row r="58" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="9">
+        <v>51</v>
+      </c>
+      <c r="B58" s="23"/>
+      <c r="C58" s="23"/>
+      <c r="D58" s="23"/>
+      <c r="E58" s="22"/>
+      <c r="F58" s="23"/>
+      <c r="G58" s="22"/>
+      <c r="H58" s="22"/>
+      <c r="I58" s="22"/>
+      <c r="J58" s="22"/>
+      <c r="K58" s="22"/>
+      <c r="L58" s="22"/>
+      <c r="M58" s="22"/>
+      <c r="N58" s="22"/>
+      <c r="O58" s="23"/>
+    </row>
+    <row r="59" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="12">
+        <v>52</v>
+      </c>
+      <c r="B59" s="23"/>
+      <c r="C59" s="23"/>
+      <c r="D59" s="23"/>
+      <c r="E59" s="22"/>
+      <c r="F59" s="23"/>
+      <c r="G59" s="22"/>
+      <c r="H59" s="22"/>
+      <c r="I59" s="22"/>
+      <c r="J59" s="22"/>
+      <c r="K59" s="22"/>
+      <c r="L59" s="22"/>
+      <c r="M59" s="22"/>
+      <c r="N59" s="22"/>
+      <c r="O59" s="23"/>
+    </row>
+    <row r="60" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="9">
+        <v>53</v>
+      </c>
+      <c r="B60" s="23"/>
+      <c r="C60" s="23"/>
+      <c r="D60" s="23"/>
+      <c r="E60" s="22"/>
+      <c r="F60" s="23"/>
+      <c r="G60" s="22"/>
+      <c r="H60" s="22"/>
+      <c r="I60" s="22"/>
+      <c r="J60" s="22"/>
+      <c r="K60" s="22"/>
+      <c r="L60" s="22"/>
+      <c r="M60" s="22"/>
+      <c r="N60" s="22"/>
+      <c r="O60" s="23"/>
+    </row>
+    <row r="61" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="12">
+        <v>54</v>
+      </c>
+      <c r="B61" s="23"/>
+      <c r="C61" s="23"/>
+      <c r="D61" s="23"/>
+      <c r="E61" s="22"/>
+      <c r="F61" s="23"/>
+      <c r="G61" s="22"/>
+      <c r="H61" s="22"/>
+      <c r="I61" s="22"/>
+      <c r="J61" s="22"/>
+      <c r="K61" s="22"/>
+      <c r="L61" s="22"/>
+      <c r="M61" s="22"/>
+      <c r="N61" s="22"/>
+      <c r="O61" s="23"/>
+    </row>
+    <row r="62" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="9">
+        <v>55</v>
+      </c>
+      <c r="B62" s="23"/>
+      <c r="C62" s="23"/>
+      <c r="D62" s="23"/>
+      <c r="E62" s="22"/>
+      <c r="F62" s="23"/>
+      <c r="G62" s="22"/>
+      <c r="H62" s="22"/>
+      <c r="I62" s="22"/>
+      <c r="J62" s="22"/>
+      <c r="K62" s="22"/>
+      <c r="L62" s="22"/>
+      <c r="M62" s="22"/>
+      <c r="N62" s="22"/>
+      <c r="O62" s="23"/>
+    </row>
+    <row r="63" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="12">
+        <v>56</v>
+      </c>
+      <c r="B63" s="23"/>
+      <c r="C63" s="23"/>
+      <c r="D63" s="23"/>
+      <c r="E63" s="22"/>
+      <c r="F63" s="23"/>
+      <c r="G63" s="22"/>
+      <c r="H63" s="22"/>
+      <c r="I63" s="22"/>
+      <c r="J63" s="22"/>
+      <c r="K63" s="22"/>
+      <c r="L63" s="22"/>
+      <c r="M63" s="22"/>
+      <c r="N63" s="22"/>
+      <c r="O63" s="23"/>
+    </row>
+    <row r="64" spans="1:16" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="9">
+        <v>57</v>
+      </c>
+      <c r="B64" s="23"/>
+      <c r="C64" s="23"/>
+      <c r="D64" s="23"/>
+      <c r="E64" s="22"/>
+      <c r="F64" s="23"/>
+      <c r="G64" s="22"/>
+      <c r="H64" s="22"/>
+      <c r="I64" s="22"/>
+      <c r="J64" s="22"/>
+      <c r="K64" s="22"/>
+      <c r="L64" s="22"/>
+      <c r="M64" s="22"/>
+      <c r="N64" s="22"/>
+      <c r="O64" s="23"/>
+    </row>
+    <row r="65" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="B33" s="18"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="18"/>
-      <c r="G33" s="18"/>
-      <c r="H33" s="18"/>
-      <c r="I33" s="18"/>
-      <c r="J33" s="18"/>
-      <c r="K33" s="18"/>
-      <c r="L33" s="17">
+      <c r="B65" s="19"/>
+      <c r="C65" s="19"/>
+      <c r="D65" s="19"/>
+      <c r="E65" s="19"/>
+      <c r="F65" s="19"/>
+      <c r="G65" s="19"/>
+      <c r="H65" s="19"/>
+      <c r="I65" s="19"/>
+      <c r="J65" s="19"/>
+      <c r="K65" s="19"/>
+      <c r="L65" s="20">
         <f>IFERROR(AVERAGEIF(L10:L32,"&gt;0",L10:L32),0)</f>
         <v>1</v>
       </c>
-      <c r="M33" s="2"/>
-      <c r="N33" s="2"/>
-      <c r="O33" s="2"/>
+      <c r="M65" s="21"/>
+      <c r="N65" s="21"/>
+      <c r="O65" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -2859,7 +4137,7 @@
     <mergeCell ref="K3:O3"/>
     <mergeCell ref="B4:J4"/>
     <mergeCell ref="K4:O4"/>
-    <mergeCell ref="A33:K33"/>
+    <mergeCell ref="A65:K65"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="G6:I6"/>
     <mergeCell ref="K6:L6"/>
@@ -2887,47 +4165,47 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="7" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="7" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="7" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="7" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="7" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="7" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="7" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="7" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="7" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2950,262 +4228,262 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3"/>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
     </row>
     <row r="2" spans="1:4" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
     </row>
     <row r="3" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="31"/>
-      <c r="B3" s="12" t="s">
+      <c r="A3" s="9"/>
+      <c r="B3" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="31"/>
-      <c r="B4" s="33" t="s">
+      <c r="A4" s="9"/>
+      <c r="B4" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
     </row>
     <row r="5" spans="1:4" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
     </row>
     <row r="7" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="14" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="4" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="2" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="4" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="2" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="4" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="2" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="4" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="2" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="4" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="14" t="s">
+      <c r="C17" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="2" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="C18" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="4" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="C19" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="2" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C20" s="16" t="s">
+      <c r="C20" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="4" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="22" spans="2:4" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="34" t="s">
+      <c r="B22" s="16" t="s">
         <v>132</v>
       </c>
-      <c r="C22" s="34"/>
-      <c r="D22" s="34"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
     </row>
     <row r="24" spans="2:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="17" t="s">
         <v>133</v>
       </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
     </row>
     <row r="25" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
     </row>
     <row r="26" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
     </row>
     <row r="27" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
     </row>
     <row r="28" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
     </row>
     <row r="29" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="9" t="s">
+      <c r="B29" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
+      <c r="C29" s="7"/>
+      <c r="D29" s="7"/>
     </row>
     <row r="30" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="1" t="s">
+      <c r="B30" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
     </row>
     <row r="31" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="9" t="s">
+      <c r="B31" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
     </row>
     <row r="32" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="8" t="s">
+      <c r="B32" s="16" t="s">
         <v>141</v>
       </c>
       <c r="C32" s="7"/>

</xml_diff>